<commit_message>
Update MLB hitter fantasy scores 2026-07-11 (2026-07-10 10:54 PM)
</commit_message>
<xml_diff>
--- a/PRIZEPICKS_HITTER_AI_V3_TOP30_2026_07_11.xlsx
+++ b/PRIZEPICKS_HITTER_AI_V3_TOP30_2026_07_11.xlsx
@@ -1127,22 +1127,22 @@
         <v>11.8</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>12.39</v>
+        <v>12.41</v>
       </c>
       <c r="L2" s="5" t="n">
         <v>89.2</v>
       </c>
       <c r="M2" s="5" t="n">
-        <v>81.8</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="N2" s="5" t="n">
-        <v>81.8</v>
+        <v>81.90000000000001</v>
       </c>
       <c r="O2" s="5" t="n">
-        <v>79.90000000000001</v>
+        <v>80</v>
       </c>
       <c r="P2" s="5" t="n">
-        <v>79.90000000000001</v>
+        <v>80</v>
       </c>
       <c r="Q2" s="5" t="n">
         <v>71.2</v>
@@ -1163,19 +1163,19 @@
         <v>61.9</v>
       </c>
       <c r="W2" s="6" t="n">
-        <v>56.9</v>
+        <v>57</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>56.9</v>
+        <v>57</v>
       </c>
       <c r="Y2" s="7" t="n">
-        <v>54</v>
+        <v>54.1</v>
       </c>
       <c r="Z2" s="7" t="n">
-        <v>54</v>
+        <v>54.1</v>
       </c>
       <c r="AA2" s="3" t="n">
-        <v>294.79</v>
+        <v>294.94</v>
       </c>
       <c r="AB2" s="4" t="inlineStr">
         <is>
@@ -1239,7 +1239,7 @@
         <v>0.2557</v>
       </c>
       <c r="AS2" s="3" t="n">
-        <v>0.0347</v>
+        <v>0.0346</v>
       </c>
       <c r="AT2" s="4" t="inlineStr">
         <is>
@@ -1253,13 +1253,13 @@
         <v>1.01</v>
       </c>
       <c r="AW2" s="3" t="n">
-        <v>71.90000000000001</v>
+        <v>72.3</v>
       </c>
       <c r="AX2" s="3" t="n">
-        <v>11</v>
+        <v>11.2</v>
       </c>
       <c r="AY2" s="3" t="n">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AZ2" s="3" t="n">
         <v>1</v>
@@ -1375,7 +1375,7 @@
         <v>0.0646</v>
       </c>
       <c r="CK2" s="3" t="n">
-        <v>0.0672</v>
+        <v>0.0674</v>
       </c>
       <c r="CL2" s="3" t="n">
         <v>0.0056</v>
@@ -1453,10 +1453,10 @@
         <v>77</v>
       </c>
       <c r="O3" s="5" t="n">
-        <v>73.90000000000001</v>
+        <v>73.8</v>
       </c>
       <c r="P3" s="5" t="n">
-        <v>73.90000000000001</v>
+        <v>73.8</v>
       </c>
       <c r="Q3" s="5" t="n">
         <v>64.8</v>
@@ -1567,13 +1567,13 @@
         <v>1.03</v>
       </c>
       <c r="AW3" s="3" t="n">
-        <v>85.7</v>
+        <v>84.2</v>
       </c>
       <c r="AX3" s="3" t="n">
-        <v>4.7</v>
+        <v>4.8</v>
       </c>
       <c r="AY3" s="3" t="n">
-        <v>355</v>
+        <v>332</v>
       </c>
       <c r="AZ3" s="3" t="n">
         <v>14</v>
@@ -1767,16 +1767,16 @@
         <v>78.7</v>
       </c>
       <c r="O4" s="5" t="n">
-        <v>74.09999999999999</v>
+        <v>74</v>
       </c>
       <c r="P4" s="5" t="n">
-        <v>74.09999999999999</v>
+        <v>74</v>
       </c>
       <c r="Q4" s="5" t="n">
-        <v>65.09999999999999</v>
+        <v>65.2</v>
       </c>
       <c r="R4" s="5" t="n">
-        <v>65.09999999999999</v>
+        <v>65.2</v>
       </c>
       <c r="S4" s="5" t="n">
         <v>61.4</v>
@@ -1785,16 +1785,16 @@
         <v>61.4</v>
       </c>
       <c r="U4" s="6" t="n">
-        <v>54.6</v>
+        <v>54.7</v>
       </c>
       <c r="V4" s="7" t="n">
-        <v>54.6</v>
+        <v>54.7</v>
       </c>
       <c r="W4" s="7" t="n">
-        <v>49.8</v>
+        <v>49.9</v>
       </c>
       <c r="X4" s="7" t="n">
-        <v>49.8</v>
+        <v>49.9</v>
       </c>
       <c r="Y4" s="7" t="n">
         <v>45.7</v>
@@ -1803,7 +1803,7 @@
         <v>45.7</v>
       </c>
       <c r="AA4" s="3" t="n">
-        <v>276.98</v>
+        <v>277.01</v>
       </c>
       <c r="AB4" s="4" t="inlineStr">
         <is>
@@ -2066,25 +2066,25 @@
         </is>
       </c>
       <c r="J5" s="3" t="n">
-        <v>11.18</v>
+        <v>11.17</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>11.54</v>
+        <v>11.48</v>
       </c>
       <c r="L5" s="5" t="n">
-        <v>91.90000000000001</v>
+        <v>91.7</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>83.09999999999999</v>
+        <v>83</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>83.09999999999999</v>
+        <v>83</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>82.3</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="P5" s="5" t="n">
-        <v>82.3</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="Q5" s="5" t="n">
         <v>73.5</v>
@@ -2093,31 +2093,31 @@
         <v>73.5</v>
       </c>
       <c r="S5" s="5" t="n">
-        <v>68.7</v>
+        <v>68.5</v>
       </c>
       <c r="T5" s="5" t="n">
-        <v>68.7</v>
+        <v>68.5</v>
       </c>
       <c r="U5" s="5" t="n">
-        <v>64.2</v>
+        <v>63.8</v>
       </c>
       <c r="V5" s="5" t="n">
-        <v>64.2</v>
+        <v>63.8</v>
       </c>
       <c r="W5" s="6" t="n">
-        <v>56.5</v>
+        <v>56.2</v>
       </c>
       <c r="X5" s="7" t="n">
-        <v>56.5</v>
+        <v>56.2</v>
       </c>
       <c r="Y5" s="7" t="n">
-        <v>53.6</v>
+        <v>53.2</v>
       </c>
       <c r="Z5" s="7" t="n">
-        <v>53.6</v>
+        <v>53.2</v>
       </c>
       <c r="AA5" s="3" t="n">
-        <v>273.38</v>
+        <v>273.31</v>
       </c>
       <c r="AB5" s="4" t="inlineStr">
         <is>
@@ -2181,7 +2181,7 @@
         <v>0.2557</v>
       </c>
       <c r="AS5" s="3" t="n">
-        <v>0.0347</v>
+        <v>0.0346</v>
       </c>
       <c r="AT5" s="4" t="inlineStr">
         <is>
@@ -2195,13 +2195,13 @@
         <v>1.01</v>
       </c>
       <c r="AW5" s="3" t="n">
-        <v>71.90000000000001</v>
+        <v>72.3</v>
       </c>
       <c r="AX5" s="3" t="n">
-        <v>11</v>
+        <v>11.2</v>
       </c>
       <c r="AY5" s="3" t="n">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AZ5" s="3" t="n">
         <v>1</v>
@@ -2212,7 +2212,7 @@
         </is>
       </c>
       <c r="BB5" s="3" t="n">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="BC5" s="3" t="n">
         <v>354</v>
@@ -2221,13 +2221,13 @@
         <v>0.331</v>
       </c>
       <c r="BE5" s="3" t="n">
-        <v>0.367</v>
+        <v>0.369</v>
       </c>
       <c r="BF5" s="3" t="n">
         <v>0.463</v>
       </c>
       <c r="BG5" s="3" t="n">
-        <v>0.83</v>
+        <v>0.832</v>
       </c>
       <c r="BH5" s="3" t="n">
         <v>118</v>
@@ -2254,7 +2254,7 @@
         <v>35</v>
       </c>
       <c r="BP5" s="3" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="BQ5" s="3" t="n">
         <v>3</v>
@@ -2263,37 +2263,37 @@
         <v>8</v>
       </c>
       <c r="BS5" s="3" t="n">
-        <v>9.289999999999999</v>
+        <v>9.57</v>
       </c>
       <c r="BT5" s="3" t="n">
-        <v>9.07</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="BU5" s="3" t="n">
-        <v>8.83</v>
+        <v>8.9</v>
       </c>
       <c r="BV5" s="3" t="n">
-        <v>2.082</v>
+        <v>2.081</v>
       </c>
       <c r="BW5" s="3" t="n">
-        <v>0.3443</v>
+        <v>0.3387</v>
       </c>
       <c r="BX5" s="3" t="n">
-        <v>0.1148</v>
+        <v>0.1129</v>
       </c>
       <c r="BY5" s="3" t="n">
-        <v>0.0164</v>
+        <v>0.0161</v>
       </c>
       <c r="BZ5" s="3" t="n">
-        <v>0.06560000000000001</v>
+        <v>0.0806</v>
       </c>
       <c r="CA5" s="3" t="n">
-        <v>0.0328</v>
+        <v>0.0323</v>
       </c>
       <c r="CB5" s="3" t="n">
         <v>10</v>
       </c>
       <c r="CC5" s="3" t="n">
-        <v>8.039999999999999</v>
+        <v>8.02</v>
       </c>
       <c r="CD5" s="3" t="n">
         <v>5</v>
@@ -2305,31 +2305,31 @@
         <v>23</v>
       </c>
       <c r="CG5" s="3" t="n">
-        <v>0.2613</v>
+        <v>0.2607</v>
       </c>
       <c r="CH5" s="3" t="n">
-        <v>0.0712</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="CI5" s="3" t="n">
         <v>0.012</v>
       </c>
       <c r="CJ5" s="3" t="n">
-        <v>0.0308</v>
+        <v>0.0307</v>
       </c>
       <c r="CK5" s="3" t="n">
-        <v>0.0481</v>
+        <v>0.0499</v>
       </c>
       <c r="CL5" s="3" t="n">
         <v>0.0068</v>
       </c>
       <c r="CM5" s="3" t="n">
-        <v>0.1361</v>
+        <v>0.1358</v>
       </c>
       <c r="CN5" s="3" t="n">
-        <v>0.1112</v>
+        <v>0.1109</v>
       </c>
       <c r="CO5" s="3" t="n">
-        <v>0.0156</v>
+        <v>0.0155</v>
       </c>
       <c r="CP5" s="4" t="inlineStr">
         <is>
@@ -2509,13 +2509,13 @@
         <v>1.03</v>
       </c>
       <c r="AW6" s="3" t="n">
-        <v>88.8</v>
+        <v>88.3</v>
       </c>
       <c r="AX6" s="3" t="n">
-        <v>5</v>
+        <v>5.9</v>
       </c>
       <c r="AY6" s="3" t="n">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="AZ6" s="3" t="n">
         <v>1</v>
@@ -2823,13 +2823,13 @@
         <v>1.03</v>
       </c>
       <c r="AW7" s="3" t="n">
-        <v>88.8</v>
+        <v>88.3</v>
       </c>
       <c r="AX7" s="3" t="n">
-        <v>5</v>
+        <v>5.9</v>
       </c>
       <c r="AY7" s="3" t="n">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="AZ7" s="3" t="n">
         <v>1</v>
@@ -3451,13 +3451,13 @@
         <v>1.01</v>
       </c>
       <c r="AW9" s="3" t="n">
-        <v>71.90000000000001</v>
+        <v>72.3</v>
       </c>
       <c r="AX9" s="3" t="n">
-        <v>11</v>
+        <v>11.2</v>
       </c>
       <c r="AY9" s="3" t="n">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AZ9" s="3" t="n">
         <v>1</v>
@@ -3765,13 +3765,13 @@
         <v>1.03</v>
       </c>
       <c r="AW10" s="3" t="n">
-        <v>88.8</v>
+        <v>88.3</v>
       </c>
       <c r="AX10" s="3" t="n">
-        <v>5</v>
+        <v>5.9</v>
       </c>
       <c r="AY10" s="3" t="n">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="AZ10" s="3" t="n">
         <v>1</v>
@@ -4079,13 +4079,13 @@
         <v>1.01</v>
       </c>
       <c r="AW11" s="3" t="n">
-        <v>71.90000000000001</v>
+        <v>72.3</v>
       </c>
       <c r="AX11" s="3" t="n">
-        <v>11</v>
+        <v>11.2</v>
       </c>
       <c r="AY11" s="3" t="n">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AZ11" s="3" t="n">
         <v>1</v>
@@ -4267,10 +4267,10 @@
         <v>10.32</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>10.2</v>
+        <v>10.19</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>83</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="M12" s="5" t="n">
         <v>75.59999999999999</v>
@@ -4279,28 +4279,28 @@
         <v>75.59999999999999</v>
       </c>
       <c r="O12" s="5" t="n">
-        <v>70.8</v>
+        <v>70.7</v>
       </c>
       <c r="P12" s="5" t="n">
-        <v>70.8</v>
+        <v>70.7</v>
       </c>
       <c r="Q12" s="5" t="n">
-        <v>61.9</v>
+        <v>61.8</v>
       </c>
       <c r="R12" s="5" t="n">
-        <v>61.9</v>
+        <v>61.8</v>
       </c>
       <c r="S12" s="6" t="n">
-        <v>57.9</v>
+        <v>57.8</v>
       </c>
       <c r="T12" s="7" t="n">
-        <v>57.9</v>
+        <v>57.8</v>
       </c>
       <c r="U12" s="7" t="n">
-        <v>50.9</v>
+        <v>50.8</v>
       </c>
       <c r="V12" s="7" t="n">
-        <v>50.9</v>
+        <v>50.8</v>
       </c>
       <c r="W12" s="7" t="n">
         <v>46.3</v>
@@ -4315,7 +4315,7 @@
         <v>42.6</v>
       </c>
       <c r="AA12" s="3" t="n">
-        <v>250.22</v>
+        <v>250.13</v>
       </c>
       <c r="AB12" s="4" t="inlineStr">
         <is>
@@ -4483,7 +4483,7 @@
         <v>8</v>
       </c>
       <c r="CC12" s="3" t="n">
-        <v>8.460000000000001</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="CD12" s="3" t="n">
         <v>4</v>
@@ -4541,22 +4541,22 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Casey Schmitt</t>
+          <t>Otto Lopez</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>COL @ SF</t>
+          <t>CLE @ MIA</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -4566,62 +4566,62 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>LF</t>
+          <t>SS</t>
         </is>
       </c>
       <c r="J13" s="3" t="n">
-        <v>10.93</v>
+        <v>9.81</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>10.91</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="L13" s="5" t="n">
-        <v>87.8</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>77.59999999999999</v>
+        <v>73.2</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>77.59999999999999</v>
+        <v>73.2</v>
       </c>
       <c r="O13" s="5" t="n">
-        <v>76.40000000000001</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="P13" s="5" t="n">
-        <v>76.40000000000001</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="Q13" s="5" t="n">
-        <v>66.8</v>
+        <v>60</v>
       </c>
       <c r="R13" s="5" t="n">
-        <v>66.8</v>
-      </c>
-      <c r="S13" s="5" t="n">
-        <v>61.8</v>
-      </c>
-      <c r="T13" s="5" t="n">
-        <v>61.8</v>
-      </c>
-      <c r="U13" s="6" t="n">
-        <v>57</v>
+        <v>60</v>
+      </c>
+      <c r="S13" s="6" t="n">
+        <v>56.6</v>
+      </c>
+      <c r="T13" s="7" t="n">
+        <v>56.6</v>
+      </c>
+      <c r="U13" s="7" t="n">
+        <v>50.4</v>
       </c>
       <c r="V13" s="7" t="n">
-        <v>57</v>
+        <v>50.4</v>
       </c>
       <c r="W13" s="7" t="n">
-        <v>50.1</v>
+        <v>44.6</v>
       </c>
       <c r="X13" s="7" t="n">
-        <v>50.1</v>
+        <v>44.6</v>
       </c>
       <c r="Y13" s="7" t="n">
-        <v>47.7</v>
+        <v>41.5</v>
       </c>
       <c r="Z13" s="7" t="n">
-        <v>47.7</v>
+        <v>41.5</v>
       </c>
       <c r="AA13" s="3" t="n">
-        <v>249.37</v>
+        <v>249.32</v>
       </c>
       <c r="AB13" s="4" t="inlineStr">
         <is>
@@ -4630,14 +4630,14 @@
       </c>
       <c r="AC13" s="8" t="inlineStr">
         <is>
-          <t>Forecast 10.9 FS | Sim 10.9</t>
+          <t>Forecast 9.8 FS | Sim 9.5</t>
         </is>
       </c>
       <c r="AD13" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AE13" s="3" t="n">
-        <v>4.82</v>
+        <v>5.13</v>
       </c>
       <c r="AF13" s="4" t="inlineStr">
         <is>
@@ -4645,199 +4645,191 @@
         </is>
       </c>
       <c r="AG13" s="3" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AH13" s="3" t="n">
         <v>1.04</v>
       </c>
       <c r="AI13" s="4" t="inlineStr">
         <is>
-          <t>Kyle Freeland</t>
+          <t>Tanner Bibee</t>
         </is>
       </c>
       <c r="AJ13" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>R</t>
         </is>
       </c>
       <c r="AK13" s="3" t="n">
-        <v>7.46</v>
+        <v>4.06</v>
       </c>
       <c r="AL13" s="3" t="n">
-        <v>1.61</v>
+        <v>1.14</v>
       </c>
       <c r="AM13" s="3" t="n">
-        <v>0.3016</v>
+        <v>0.2116</v>
       </c>
       <c r="AN13" s="3" t="n">
-        <v>0.045</v>
+        <v>0.0465</v>
       </c>
       <c r="AO13" s="3" t="n">
-        <v>0.0476</v>
+        <v>0.0698</v>
       </c>
       <c r="AP13" s="3" t="n">
-        <v>5.46</v>
+        <v>3.76</v>
       </c>
       <c r="AQ13" s="3" t="n">
-        <v>1.52</v>
+        <v>1.26</v>
       </c>
       <c r="AR13" s="3" t="n">
-        <v>0.2557</v>
+        <v>0.211</v>
       </c>
       <c r="AS13" s="3" t="n">
-        <v>0.0347</v>
+        <v>0.0308</v>
       </c>
       <c r="AT13" s="4" t="inlineStr">
         <is>
-          <t>Oracle Park</t>
+          <t>loanDepot park</t>
         </is>
       </c>
       <c r="AU13" s="3" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.96</v>
       </c>
       <c r="AV13" s="3" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="AW13" s="3" t="n">
-        <v>71.90000000000001</v>
-      </c>
-      <c r="AX13" s="3" t="n">
-        <v>11</v>
-      </c>
-      <c r="AY13" s="3" t="n">
-        <v>274</v>
-      </c>
-      <c r="AZ13" s="3" t="n">
         <v>1</v>
       </c>
+      <c r="AW13" s="4" t="n"/>
+      <c r="AX13" s="4" t="n"/>
+      <c r="AY13" s="4" t="n"/>
+      <c r="AZ13" s="4" t="n"/>
       <c r="BA13" s="4" t="inlineStr">
         <is>
-          <t>light wind</t>
+          <t>Indoor/retractable neutral</t>
         </is>
       </c>
       <c r="BB13" s="3" t="n">
-        <v>361</v>
+        <v>401</v>
       </c>
       <c r="BC13" s="3" t="n">
-        <v>341</v>
+        <v>372</v>
       </c>
       <c r="BD13" s="3" t="n">
-        <v>0.279</v>
+        <v>0.341</v>
       </c>
       <c r="BE13" s="3" t="n">
-        <v>0.307</v>
+        <v>0.374</v>
       </c>
       <c r="BF13" s="3" t="n">
-        <v>0.493</v>
+        <v>0.516</v>
       </c>
       <c r="BG13" s="3" t="n">
-        <v>0.8</v>
+        <v>0.89</v>
       </c>
       <c r="BH13" s="3" t="n">
-        <v>97</v>
+        <v>309</v>
       </c>
       <c r="BI13" s="3" t="n">
-        <v>0.829</v>
+        <v>0.835</v>
       </c>
       <c r="BJ13" s="3" t="n">
-        <v>95</v>
+        <v>127</v>
       </c>
       <c r="BK13" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="BL13" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="BM13" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="BN13" s="3" t="n">
+        <v>61</v>
+      </c>
+      <c r="BO13" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="BP13" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="BQ13" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="BR13" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="BL13" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="BM13" s="3" t="n">
-        <v>18</v>
-      </c>
-      <c r="BN13" s="3" t="n">
-        <v>41</v>
-      </c>
-      <c r="BO13" s="3" t="n">
-        <v>47</v>
-      </c>
-      <c r="BP13" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="BQ13" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="BR13" s="3" t="n">
-        <v>7</v>
-      </c>
       <c r="BS13" s="3" t="n">
-        <v>8.43</v>
+        <v>14.29</v>
       </c>
       <c r="BT13" s="3" t="n">
-        <v>5.43</v>
+        <v>12.86</v>
       </c>
       <c r="BU13" s="3" t="n">
-        <v>5.9</v>
+        <v>11.6</v>
       </c>
       <c r="BV13" s="3" t="n">
-        <v>1.357</v>
+        <v>2.769</v>
       </c>
       <c r="BW13" s="3" t="n">
-        <v>0.1786</v>
+        <v>0.3385</v>
       </c>
       <c r="BX13" s="3" t="n">
-        <v>0.07140000000000001</v>
+        <v>0.1846</v>
       </c>
       <c r="BY13" s="3" t="n">
-        <v>0.0357</v>
+        <v>0.0615</v>
       </c>
       <c r="BZ13" s="3" t="n">
-        <v>0.0357</v>
+        <v>0.0615</v>
       </c>
       <c r="CA13" s="3" t="n">
-        <v>0</v>
+        <v>0.0154</v>
       </c>
       <c r="CB13" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="CC13" s="3" t="n">
-        <v>8.56</v>
+        <v>7.91</v>
       </c>
       <c r="CD13" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="CE13" s="3" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="CF13" s="3" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="CG13" s="3" t="n">
-        <v>0.223</v>
+        <v>0.1641</v>
       </c>
       <c r="CH13" s="3" t="n">
-        <v>0.0626</v>
+        <v>0.0508</v>
       </c>
       <c r="CI13" s="3" t="n">
-        <v>0.0044</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="CJ13" s="3" t="n">
-        <v>0.0527</v>
+        <v>0.0377</v>
       </c>
       <c r="CK13" s="3" t="n">
-        <v>0.0386</v>
+        <v>0.0594</v>
       </c>
       <c r="CL13" s="3" t="n">
-        <v>0.0095</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="CM13" s="3" t="n">
-        <v>0.1263</v>
+        <v>0.1377</v>
       </c>
       <c r="CN13" s="3" t="n">
-        <v>0.155</v>
+        <v>0.1015</v>
       </c>
       <c r="CO13" s="3" t="n">
-        <v>0.0132</v>
+        <v>0.0206</v>
       </c>
       <c r="CP13" s="4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -4855,22 +4847,22 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Otto Lopez</t>
+          <t>Casey Schmitt</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>CLE @ MIA</t>
+          <t>COL @ SF</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
@@ -4880,62 +4872,62 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>LF</t>
         </is>
       </c>
       <c r="J14" s="3" t="n">
-        <v>9.81</v>
+        <v>10.92</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>9.529999999999999</v>
+        <v>10.91</v>
       </c>
       <c r="L14" s="5" t="n">
-        <v>82.90000000000001</v>
+        <v>87.8</v>
       </c>
       <c r="M14" s="5" t="n">
-        <v>73.2</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="N14" s="5" t="n">
-        <v>73.2</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="O14" s="5" t="n">
-        <v>70.59999999999999</v>
+        <v>76.3</v>
       </c>
       <c r="P14" s="5" t="n">
-        <v>70.59999999999999</v>
+        <v>76.3</v>
       </c>
       <c r="Q14" s="5" t="n">
-        <v>60</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="R14" s="5" t="n">
-        <v>60</v>
-      </c>
-      <c r="S14" s="6" t="n">
-        <v>56.6</v>
-      </c>
-      <c r="T14" s="7" t="n">
-        <v>56.6</v>
-      </c>
-      <c r="U14" s="7" t="n">
-        <v>50.4</v>
+        <v>66.59999999999999</v>
+      </c>
+      <c r="S14" s="5" t="n">
+        <v>61.7</v>
+      </c>
+      <c r="T14" s="5" t="n">
+        <v>61.7</v>
+      </c>
+      <c r="U14" s="6" t="n">
+        <v>57</v>
       </c>
       <c r="V14" s="7" t="n">
-        <v>50.4</v>
+        <v>57</v>
       </c>
       <c r="W14" s="7" t="n">
-        <v>44.6</v>
+        <v>50.2</v>
       </c>
       <c r="X14" s="7" t="n">
-        <v>44.6</v>
+        <v>50.2</v>
       </c>
       <c r="Y14" s="7" t="n">
-        <v>41.5</v>
+        <v>47.8</v>
       </c>
       <c r="Z14" s="7" t="n">
-        <v>41.5</v>
+        <v>47.8</v>
       </c>
       <c r="AA14" s="3" t="n">
-        <v>249.25</v>
+        <v>249.28</v>
       </c>
       <c r="AB14" s="4" t="inlineStr">
         <is>
@@ -4944,14 +4936,14 @@
       </c>
       <c r="AC14" s="8" t="inlineStr">
         <is>
-          <t>Forecast 9.8 FS | Sim 9.5</t>
+          <t>Forecast 10.9 FS | Sim 10.9</t>
         </is>
       </c>
       <c r="AD14" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="AE14" s="3" t="n">
-        <v>5.13</v>
+        <v>4.82</v>
       </c>
       <c r="AF14" s="4" t="inlineStr">
         <is>
@@ -4959,191 +4951,199 @@
         </is>
       </c>
       <c r="AG14" s="3" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AH14" s="3" t="n">
         <v>1.04</v>
       </c>
       <c r="AI14" s="4" t="inlineStr">
         <is>
-          <t>Tanner Bibee</t>
+          <t>Kyle Freeland</t>
         </is>
       </c>
       <c r="AJ14" s="4" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>L</t>
         </is>
       </c>
       <c r="AK14" s="3" t="n">
-        <v>4.06</v>
+        <v>7.46</v>
       </c>
       <c r="AL14" s="3" t="n">
-        <v>1.14</v>
+        <v>1.61</v>
       </c>
       <c r="AM14" s="3" t="n">
-        <v>0.2116</v>
+        <v>0.3016</v>
       </c>
       <c r="AN14" s="3" t="n">
-        <v>0.0465</v>
+        <v>0.045</v>
       </c>
       <c r="AO14" s="3" t="n">
-        <v>0.0698</v>
+        <v>0.0476</v>
       </c>
       <c r="AP14" s="3" t="n">
-        <v>3.76</v>
+        <v>5.46</v>
       </c>
       <c r="AQ14" s="3" t="n">
-        <v>1.26</v>
+        <v>1.52</v>
       </c>
       <c r="AR14" s="3" t="n">
-        <v>0.211</v>
+        <v>0.2557</v>
       </c>
       <c r="AS14" s="3" t="n">
-        <v>0.0308</v>
+        <v>0.0346</v>
       </c>
       <c r="AT14" s="4" t="inlineStr">
         <is>
-          <t>loanDepot park</t>
+          <t>Oracle Park</t>
         </is>
       </c>
       <c r="AU14" s="3" t="n">
-        <v>0.96</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="AV14" s="3" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="AW14" s="3" t="n">
+        <v>72.3</v>
+      </c>
+      <c r="AX14" s="3" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="AY14" s="3" t="n">
+        <v>275</v>
+      </c>
+      <c r="AZ14" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="AW14" s="4" t="n"/>
-      <c r="AX14" s="4" t="n"/>
-      <c r="AY14" s="4" t="n"/>
-      <c r="AZ14" s="4" t="n"/>
       <c r="BA14" s="4" t="inlineStr">
         <is>
-          <t>Indoor/retractable neutral</t>
+          <t>light wind</t>
         </is>
       </c>
       <c r="BB14" s="3" t="n">
-        <v>401</v>
+        <v>362</v>
       </c>
       <c r="BC14" s="3" t="n">
-        <v>372</v>
+        <v>342</v>
       </c>
       <c r="BD14" s="3" t="n">
-        <v>0.341</v>
+        <v>0.278</v>
       </c>
       <c r="BE14" s="3" t="n">
-        <v>0.374</v>
+        <v>0.307</v>
       </c>
       <c r="BF14" s="3" t="n">
-        <v>0.516</v>
+        <v>0.491</v>
       </c>
       <c r="BG14" s="3" t="n">
-        <v>0.89</v>
+        <v>0.798</v>
       </c>
       <c r="BH14" s="3" t="n">
-        <v>309</v>
+        <v>97</v>
       </c>
       <c r="BI14" s="3" t="n">
-        <v>0.835</v>
+        <v>0.829</v>
       </c>
       <c r="BJ14" s="3" t="n">
-        <v>127</v>
+        <v>95</v>
       </c>
       <c r="BK14" s="3" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="BL14" s="3" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="BM14" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="BN14" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="BO14" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="BP14" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="BN14" s="3" t="n">
-        <v>61</v>
-      </c>
-      <c r="BO14" s="3" t="n">
-        <v>45</v>
-      </c>
-      <c r="BP14" s="3" t="n">
-        <v>19</v>
-      </c>
       <c r="BQ14" s="3" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="BR14" s="3" t="n">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="BS14" s="3" t="n">
-        <v>14.29</v>
+        <v>8.43</v>
       </c>
       <c r="BT14" s="3" t="n">
-        <v>12.86</v>
+        <v>5.43</v>
       </c>
       <c r="BU14" s="3" t="n">
-        <v>11.6</v>
+        <v>5.9</v>
       </c>
       <c r="BV14" s="3" t="n">
-        <v>2.769</v>
+        <v>1.357</v>
       </c>
       <c r="BW14" s="3" t="n">
-        <v>0.3385</v>
+        <v>0.1786</v>
       </c>
       <c r="BX14" s="3" t="n">
-        <v>0.1846</v>
+        <v>0.07140000000000001</v>
       </c>
       <c r="BY14" s="3" t="n">
-        <v>0.0615</v>
+        <v>0.0357</v>
       </c>
       <c r="BZ14" s="3" t="n">
-        <v>0.0615</v>
+        <v>0.0357</v>
       </c>
       <c r="CA14" s="3" t="n">
-        <v>0.0154</v>
+        <v>0</v>
       </c>
       <c r="CB14" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="CC14" s="3" t="n">
-        <v>7.9</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="CD14" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="CE14" s="3" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="CF14" s="3" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="CG14" s="3" t="n">
-        <v>0.1641</v>
+        <v>0.2228</v>
       </c>
       <c r="CH14" s="3" t="n">
-        <v>0.0508</v>
+        <v>0.0626</v>
       </c>
       <c r="CI14" s="3" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.0044</v>
       </c>
       <c r="CJ14" s="3" t="n">
-        <v>0.0377</v>
+        <v>0.0526</v>
       </c>
       <c r="CK14" s="3" t="n">
-        <v>0.0594</v>
+        <v>0.0387</v>
       </c>
       <c r="CL14" s="3" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="CM14" s="3" t="n">
-        <v>0.1377</v>
+        <v>0.1262</v>
       </c>
       <c r="CN14" s="3" t="n">
-        <v>0.1015</v>
+        <v>0.1549</v>
       </c>
       <c r="CO14" s="3" t="n">
-        <v>0.0206</v>
+        <v>0.0132</v>
       </c>
       <c r="CP14" s="4" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -5193,46 +5193,46 @@
         <v>10.47</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>10.41</v>
+        <v>10.42</v>
       </c>
       <c r="L15" s="5" t="n">
         <v>80.59999999999999</v>
       </c>
       <c r="M15" s="5" t="n">
-        <v>72.5</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="N15" s="5" t="n">
-        <v>72.5</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="O15" s="5" t="n">
-        <v>68.90000000000001</v>
+        <v>69</v>
       </c>
       <c r="P15" s="5" t="n">
-        <v>68.90000000000001</v>
+        <v>69</v>
       </c>
       <c r="Q15" s="5" t="n">
-        <v>59.4</v>
+        <v>59.5</v>
       </c>
       <c r="R15" s="5" t="n">
-        <v>59.4</v>
+        <v>59.5</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>56.4</v>
+        <v>56.5</v>
       </c>
       <c r="T15" s="7" t="n">
-        <v>56.4</v>
+        <v>56.5</v>
       </c>
       <c r="U15" s="7" t="n">
-        <v>50.3</v>
+        <v>50.4</v>
       </c>
       <c r="V15" s="7" t="n">
-        <v>50.3</v>
+        <v>50.4</v>
       </c>
       <c r="W15" s="7" t="n">
-        <v>46.7</v>
+        <v>46.8</v>
       </c>
       <c r="X15" s="7" t="n">
-        <v>46.7</v>
+        <v>46.8</v>
       </c>
       <c r="Y15" s="7" t="n">
         <v>43.8</v>
@@ -5241,7 +5241,7 @@
         <v>43.8</v>
       </c>
       <c r="AA15" s="3" t="n">
-        <v>248.85</v>
+        <v>248.96</v>
       </c>
       <c r="AB15" s="4" t="inlineStr">
         <is>
@@ -5507,22 +5507,22 @@
         <v>10.48</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>10.55</v>
+        <v>10.54</v>
       </c>
       <c r="L16" s="5" t="n">
-        <v>85.8</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="M16" s="5" t="n">
-        <v>76.5</v>
+        <v>76.7</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>76.5</v>
+        <v>76.7</v>
       </c>
       <c r="O16" s="5" t="n">
-        <v>74.8</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="P16" s="5" t="n">
-        <v>74.8</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="Q16" s="5" t="n">
         <v>64.5</v>
@@ -5555,7 +5555,7 @@
         <v>45.9</v>
       </c>
       <c r="AA16" s="3" t="n">
-        <v>248.82</v>
+        <v>248.75</v>
       </c>
       <c r="AB16" s="4" t="inlineStr">
         <is>
@@ -5564,7 +5564,7 @@
       </c>
       <c r="AC16" s="8" t="inlineStr">
         <is>
-          <t>Forecast 10.5 FS | Sim 10.6</t>
+          <t>Forecast 10.5 FS | Sim 10.5</t>
         </is>
       </c>
       <c r="AD16" s="3" t="n">
@@ -5619,7 +5619,7 @@
         <v>0.2557</v>
       </c>
       <c r="AS16" s="3" t="n">
-        <v>0.0347</v>
+        <v>0.0346</v>
       </c>
       <c r="AT16" s="4" t="inlineStr">
         <is>
@@ -5633,13 +5633,13 @@
         <v>1.01</v>
       </c>
       <c r="AW16" s="3" t="n">
-        <v>71.90000000000001</v>
+        <v>72.3</v>
       </c>
       <c r="AX16" s="3" t="n">
-        <v>11</v>
+        <v>11.2</v>
       </c>
       <c r="AY16" s="3" t="n">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AZ16" s="3" t="n">
         <v>1</v>
@@ -5731,7 +5731,7 @@
         <v>8</v>
       </c>
       <c r="CC16" s="3" t="n">
-        <v>8.42</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="CD16" s="3" t="n">
         <v>4</v>
@@ -5755,7 +5755,7 @@
         <v>0.0507</v>
       </c>
       <c r="CK16" s="3" t="n">
-        <v>0.0585</v>
+        <v>0.0586</v>
       </c>
       <c r="CL16" s="3" t="n">
         <v>0.0054</v>
@@ -5947,13 +5947,13 @@
         <v>1.03</v>
       </c>
       <c r="AW17" s="3" t="n">
-        <v>85.7</v>
+        <v>84.2</v>
       </c>
       <c r="AX17" s="3" t="n">
-        <v>4.7</v>
+        <v>4.8</v>
       </c>
       <c r="AY17" s="3" t="n">
-        <v>355</v>
+        <v>332</v>
       </c>
       <c r="AZ17" s="3" t="n">
         <v>14</v>
@@ -6444,13 +6444,13 @@
         <v>10.02</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>82.90000000000001</v>
+        <v>83</v>
       </c>
       <c r="M19" s="5" t="n">
-        <v>75.59999999999999</v>
+        <v>75.7</v>
       </c>
       <c r="N19" s="5" t="n">
-        <v>75.59999999999999</v>
+        <v>75.7</v>
       </c>
       <c r="O19" s="5" t="n">
         <v>71</v>
@@ -6459,10 +6459,10 @@
         <v>71</v>
       </c>
       <c r="Q19" s="5" t="n">
-        <v>61.4</v>
+        <v>61.5</v>
       </c>
       <c r="R19" s="5" t="n">
-        <v>61.4</v>
+        <v>61.5</v>
       </c>
       <c r="S19" s="6" t="n">
         <v>57.3</v>
@@ -6657,7 +6657,7 @@
         <v>7</v>
       </c>
       <c r="CC19" s="3" t="n">
-        <v>8.380000000000001</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="CD19" s="3" t="n">
         <v>4</v>
@@ -6747,7 +6747,7 @@
         <v>9.800000000000001</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>9.51</v>
+        <v>9.5</v>
       </c>
       <c r="L20" s="5" t="n">
         <v>80.8</v>
@@ -6765,37 +6765,37 @@
         <v>68</v>
       </c>
       <c r="Q20" s="5" t="n">
-        <v>58.2</v>
+        <v>58.1</v>
       </c>
       <c r="R20" s="5" t="n">
-        <v>58.2</v>
+        <v>58.1</v>
       </c>
       <c r="S20" s="6" t="n">
-        <v>54.1</v>
+        <v>54</v>
       </c>
       <c r="T20" s="7" t="n">
-        <v>54.1</v>
+        <v>54</v>
       </c>
       <c r="U20" s="7" t="n">
-        <v>47.2</v>
+        <v>47.1</v>
       </c>
       <c r="V20" s="7" t="n">
-        <v>47.2</v>
+        <v>47.1</v>
       </c>
       <c r="W20" s="7" t="n">
-        <v>42.8</v>
+        <v>42.7</v>
       </c>
       <c r="X20" s="7" t="n">
-        <v>42.8</v>
+        <v>42.7</v>
       </c>
       <c r="Y20" s="9" t="n">
-        <v>39</v>
+        <v>38.9</v>
       </c>
       <c r="Z20" s="9" t="n">
-        <v>39</v>
+        <v>38.9</v>
       </c>
       <c r="AA20" s="3" t="n">
-        <v>243.12</v>
+        <v>243.01</v>
       </c>
       <c r="AB20" s="4" t="inlineStr">
         <is>
@@ -6873,13 +6873,13 @@
         <v>1.03</v>
       </c>
       <c r="AW20" s="3" t="n">
-        <v>84.3</v>
+        <v>84.8</v>
       </c>
       <c r="AX20" s="3" t="n">
-        <v>7.4</v>
+        <v>7</v>
       </c>
       <c r="AY20" s="3" t="n">
-        <v>110</v>
+        <v>81</v>
       </c>
       <c r="AZ20" s="3" t="n">
         <v>13</v>
@@ -6971,7 +6971,7 @@
         <v>7</v>
       </c>
       <c r="CC20" s="3" t="n">
-        <v>8.18</v>
+        <v>8.17</v>
       </c>
       <c r="CD20" s="3" t="n">
         <v>3</v>
@@ -7061,7 +7061,7 @@
         <v>9.789999999999999</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>9.41</v>
+        <v>9.4</v>
       </c>
       <c r="L21" s="5" t="n">
         <v>82.40000000000001</v>
@@ -7109,7 +7109,7 @@
         <v>39.9</v>
       </c>
       <c r="AA21" s="3" t="n">
-        <v>242.44</v>
+        <v>242.37</v>
       </c>
       <c r="AB21" s="4" t="inlineStr">
         <is>
@@ -7285,7 +7285,7 @@
         <v>7</v>
       </c>
       <c r="CC21" s="3" t="n">
-        <v>7.77</v>
+        <v>7.76</v>
       </c>
       <c r="CD21" s="3" t="n">
         <v>3</v>
@@ -7375,7 +7375,7 @@
         <v>9.91</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>9.99</v>
+        <v>9.98</v>
       </c>
       <c r="L22" s="5" t="n">
         <v>83.8</v>
@@ -7411,10 +7411,10 @@
         <v>51.4</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>46.4</v>
+        <v>46.3</v>
       </c>
       <c r="X22" s="7" t="n">
-        <v>46.4</v>
+        <v>46.3</v>
       </c>
       <c r="Y22" s="7" t="n">
         <v>42.7</v>
@@ -7423,7 +7423,7 @@
         <v>42.7</v>
       </c>
       <c r="AA22" s="3" t="n">
-        <v>242.36</v>
+        <v>242.28</v>
       </c>
       <c r="AB22" s="4" t="inlineStr">
         <is>
@@ -7591,7 +7591,7 @@
         <v>8</v>
       </c>
       <c r="CC22" s="3" t="n">
-        <v>8.119999999999999</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="CD22" s="3" t="n">
         <v>4</v>
@@ -7807,13 +7807,13 @@
         <v>1.01</v>
       </c>
       <c r="AW23" s="3" t="n">
-        <v>71.90000000000001</v>
+        <v>72.3</v>
       </c>
       <c r="AX23" s="3" t="n">
-        <v>11</v>
+        <v>11.2</v>
       </c>
       <c r="AY23" s="3" t="n">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AZ23" s="3" t="n">
         <v>1</v>
@@ -8031,19 +8031,19 @@
         <v>50.5</v>
       </c>
       <c r="W24" s="7" t="n">
-        <v>45.5</v>
+        <v>45.6</v>
       </c>
       <c r="X24" s="7" t="n">
-        <v>45.5</v>
+        <v>45.6</v>
       </c>
       <c r="Y24" s="7" t="n">
-        <v>42.1</v>
+        <v>42.2</v>
       </c>
       <c r="Z24" s="7" t="n">
-        <v>42.1</v>
+        <v>42.2</v>
       </c>
       <c r="AA24" s="3" t="n">
-        <v>238.51</v>
+        <v>238.52</v>
       </c>
       <c r="AB24" s="4" t="inlineStr">
         <is>
@@ -8315,49 +8315,49 @@
         <v>84.7</v>
       </c>
       <c r="M25" s="5" t="n">
-        <v>73.40000000000001</v>
+        <v>73.5</v>
       </c>
       <c r="N25" s="5" t="n">
-        <v>73.40000000000001</v>
+        <v>73.5</v>
       </c>
       <c r="O25" s="5" t="n">
-        <v>71.8</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="P25" s="5" t="n">
-        <v>71.8</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="Q25" s="5" t="n">
-        <v>60.8</v>
+        <v>60.9</v>
       </c>
       <c r="R25" s="5" t="n">
-        <v>60.8</v>
+        <v>60.9</v>
       </c>
       <c r="S25" s="6" t="n">
-        <v>56.7</v>
+        <v>56.8</v>
       </c>
       <c r="T25" s="7" t="n">
-        <v>56.7</v>
+        <v>56.8</v>
       </c>
       <c r="U25" s="7" t="n">
-        <v>51.2</v>
+        <v>51.3</v>
       </c>
       <c r="V25" s="7" t="n">
-        <v>51.2</v>
+        <v>51.3</v>
       </c>
       <c r="W25" s="7" t="n">
-        <v>45</v>
+        <v>45.1</v>
       </c>
       <c r="X25" s="7" t="n">
-        <v>45</v>
+        <v>45.1</v>
       </c>
       <c r="Y25" s="7" t="n">
-        <v>42.5</v>
+        <v>42.4</v>
       </c>
       <c r="Z25" s="7" t="n">
-        <v>42.5</v>
+        <v>42.4</v>
       </c>
       <c r="AA25" s="3" t="n">
-        <v>238.11</v>
+        <v>238.14</v>
       </c>
       <c r="AB25" s="4" t="inlineStr">
         <is>
@@ -8421,7 +8421,7 @@
         <v>0.2557</v>
       </c>
       <c r="AS25" s="3" t="n">
-        <v>0.0347</v>
+        <v>0.0346</v>
       </c>
       <c r="AT25" s="4" t="inlineStr">
         <is>
@@ -8435,13 +8435,13 @@
         <v>1.01</v>
       </c>
       <c r="AW25" s="3" t="n">
-        <v>71.90000000000001</v>
+        <v>72.3</v>
       </c>
       <c r="AX25" s="3" t="n">
-        <v>11</v>
+        <v>11.2</v>
       </c>
       <c r="AY25" s="3" t="n">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="AZ25" s="3" t="n">
         <v>1</v>
@@ -8554,13 +8554,13 @@
         <v>0.0104</v>
       </c>
       <c r="CJ25" s="3" t="n">
-        <v>0.0512</v>
+        <v>0.0511</v>
       </c>
       <c r="CK25" s="3" t="n">
-        <v>0.0497</v>
+        <v>0.0498</v>
       </c>
       <c r="CL25" s="3" t="n">
-        <v>0.0055</v>
+        <v>0.0056</v>
       </c>
       <c r="CM25" s="3" t="n">
         <v>0.1324</v>
@@ -8623,10 +8623,10 @@
         <v>9.119999999999999</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>8.890000000000001</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="L26" s="5" t="n">
-        <v>73.90000000000001</v>
+        <v>73.8</v>
       </c>
       <c r="M26" s="5" t="n">
         <v>64.5</v>
@@ -8665,13 +8665,13 @@
         <v>38.7</v>
       </c>
       <c r="Y26" s="9" t="n">
-        <v>36.4</v>
+        <v>36.3</v>
       </c>
       <c r="Z26" s="9" t="n">
-        <v>36.4</v>
+        <v>36.3</v>
       </c>
       <c r="AA26" s="3" t="n">
-        <v>236.8</v>
+        <v>236.73</v>
       </c>
       <c r="AB26" s="4" t="inlineStr">
         <is>
@@ -9055,13 +9055,13 @@
         <v>1.03</v>
       </c>
       <c r="AW27" s="3" t="n">
-        <v>83.7</v>
+        <v>82.8</v>
       </c>
       <c r="AX27" s="3" t="n">
-        <v>4.5</v>
+        <v>3.3</v>
       </c>
       <c r="AY27" s="3" t="n">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="AZ27" s="3" t="n">
         <v>10</v>
@@ -9211,22 +9211,22 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>James Wood</t>
+          <t>Trevor Larnach</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>WSH</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>NYY</t>
+          <t>LAA</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>NYY @ WSH</t>
+          <t>LAA @ MIN</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
@@ -9236,62 +9236,62 @@
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>RF</t>
+          <t>LF</t>
         </is>
       </c>
       <c r="J28" s="3" t="n">
-        <v>8.779999999999999</v>
+        <v>9.630000000000001</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>7.95</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="L28" s="5" t="n">
-        <v>72.40000000000001</v>
+        <v>85.2</v>
       </c>
       <c r="M28" s="5" t="n">
-        <v>65.40000000000001</v>
+        <v>76.8</v>
       </c>
       <c r="N28" s="5" t="n">
-        <v>65.40000000000001</v>
+        <v>76.8</v>
       </c>
       <c r="O28" s="5" t="n">
-        <v>59.6</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="P28" s="5" t="n">
-        <v>59.6</v>
-      </c>
-      <c r="Q28" s="6" t="n">
-        <v>49.3</v>
-      </c>
-      <c r="R28" s="7" t="n">
-        <v>49.3</v>
-      </c>
-      <c r="S28" s="7" t="n">
-        <v>45.8</v>
-      </c>
-      <c r="T28" s="7" t="n">
-        <v>45.8</v>
-      </c>
-      <c r="U28" s="9" t="n">
-        <v>38.7</v>
-      </c>
-      <c r="V28" s="9" t="n">
-        <v>38.7</v>
-      </c>
-      <c r="W28" s="9" t="n">
-        <v>35.4</v>
-      </c>
-      <c r="X28" s="9" t="n">
-        <v>35.4</v>
-      </c>
-      <c r="Y28" s="9" t="n">
-        <v>31.3</v>
-      </c>
-      <c r="Z28" s="9" t="n">
-        <v>31.3</v>
+        <v>73.40000000000001</v>
+      </c>
+      <c r="Q28" s="5" t="n">
+        <v>62.6</v>
+      </c>
+      <c r="R28" s="5" t="n">
+        <v>62.6</v>
+      </c>
+      <c r="S28" s="5" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="T28" s="5" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="U28" s="6" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="V28" s="7" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="W28" s="7" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="X28" s="7" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="Y28" s="7" t="n">
+        <v>41</v>
+      </c>
+      <c r="Z28" s="7" t="n">
+        <v>41</v>
       </c>
       <c r="AA28" s="3" t="n">
-        <v>234.76</v>
+        <v>234.73</v>
       </c>
       <c r="AB28" s="4" t="inlineStr">
         <is>
@@ -9300,14 +9300,14 @@
       </c>
       <c r="AC28" s="8" t="inlineStr">
         <is>
-          <t>Forecast 8.8 FS | Sim 8.0</t>
+          <t>Forecast 9.6 FS | Sim 9.7</t>
         </is>
       </c>
       <c r="AD28" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AE28" s="3" t="n">
-        <v>5.13</v>
+        <v>4.52</v>
       </c>
       <c r="AF28" s="4" t="inlineStr">
         <is>
@@ -9315,14 +9315,14 @@
         </is>
       </c>
       <c r="AG28" s="3" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="AH28" s="3" t="n">
         <v>1.04</v>
       </c>
       <c r="AI28" s="4" t="inlineStr">
         <is>
-          <t>Cam Schlittler</t>
+          <t>Ryan Johnson</t>
         </is>
       </c>
       <c r="AJ28" s="4" t="inlineStr">
@@ -9331,54 +9331,54 @@
         </is>
       </c>
       <c r="AK28" s="3" t="n">
-        <v>2.01</v>
+        <v>6.99</v>
       </c>
       <c r="AL28" s="3" t="n">
-        <v>0.93</v>
+        <v>1.55</v>
       </c>
       <c r="AM28" s="3" t="n">
-        <v>0.1878</v>
+        <v>0.2595</v>
       </c>
       <c r="AN28" s="3" t="n">
-        <v>0.0226</v>
+        <v>0.0611</v>
       </c>
       <c r="AO28" s="3" t="n">
-        <v>0.0475</v>
+        <v>0.07630000000000001</v>
       </c>
       <c r="AP28" s="3" t="n">
-        <v>3.4</v>
+        <v>4.65</v>
       </c>
       <c r="AQ28" s="3" t="n">
-        <v>1.19</v>
+        <v>1.4</v>
       </c>
       <c r="AR28" s="3" t="n">
-        <v>0.2049</v>
+        <v>0.2052</v>
       </c>
       <c r="AS28" s="3" t="n">
-        <v>0.0267</v>
+        <v>0.028</v>
       </c>
       <c r="AT28" s="4" t="inlineStr">
         <is>
-          <t>Nationals Park</t>
+          <t>Target Field</t>
         </is>
       </c>
       <c r="AU28" s="3" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="AV28" s="3" t="n">
         <v>1.03</v>
       </c>
       <c r="AW28" s="3" t="n">
-        <v>85.7</v>
+        <v>88.3</v>
       </c>
       <c r="AX28" s="3" t="n">
-        <v>4.7</v>
+        <v>5.9</v>
       </c>
       <c r="AY28" s="3" t="n">
-        <v>355</v>
+        <v>191</v>
       </c>
       <c r="AZ28" s="3" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="BA28" s="4" t="inlineStr">
         <is>
@@ -9386,128 +9386,128 @@
         </is>
       </c>
       <c r="BB28" s="3" t="n">
-        <v>445</v>
+        <v>284</v>
       </c>
       <c r="BC28" s="3" t="n">
-        <v>362</v>
+        <v>246</v>
       </c>
       <c r="BD28" s="3" t="n">
-        <v>0.273</v>
+        <v>0.285</v>
       </c>
       <c r="BE28" s="3" t="n">
-        <v>0.404</v>
+        <v>0.378</v>
       </c>
       <c r="BF28" s="3" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.439</v>
       </c>
       <c r="BG28" s="3" t="n">
-        <v>0.962</v>
+        <v>0.8169999999999999</v>
       </c>
       <c r="BH28" s="3" t="n">
-        <v>296</v>
+        <v>250</v>
       </c>
       <c r="BI28" s="3" t="n">
-        <v>0.997</v>
+        <v>0.833</v>
       </c>
       <c r="BJ28" s="3" t="n">
-        <v>99</v>
+        <v>70</v>
       </c>
       <c r="BK28" s="3" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="BL28" s="3" t="n">
         <v>1</v>
       </c>
       <c r="BM28" s="3" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="BN28" s="3" t="n">
-        <v>87</v>
+        <v>42</v>
       </c>
       <c r="BO28" s="3" t="n">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="BP28" s="3" t="n">
-        <v>77</v>
+        <v>34</v>
       </c>
       <c r="BQ28" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="BR28" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="BS28" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="BT28" s="3" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="BU28" s="3" t="n">
+        <v>7.53</v>
+      </c>
+      <c r="BV28" s="3" t="n">
+        <v>1.868</v>
+      </c>
+      <c r="BW28" s="3" t="n">
+        <v>0.2642</v>
+      </c>
+      <c r="BX28" s="3" t="n">
+        <v>0.1321</v>
+      </c>
+      <c r="BY28" s="3" t="n">
+        <v>0.0189</v>
+      </c>
+      <c r="BZ28" s="3" t="n">
+        <v>0.1132</v>
+      </c>
+      <c r="CA28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB28" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="CC28" s="3" t="n">
+        <v>7.71</v>
+      </c>
+      <c r="CD28" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="BR28" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="BS28" s="3" t="n">
-        <v>19.14</v>
-      </c>
-      <c r="BT28" s="3" t="n">
-        <v>14.86</v>
-      </c>
-      <c r="BU28" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="BV28" s="3" t="n">
-        <v>3.059</v>
-      </c>
-      <c r="BW28" s="3" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="BX28" s="3" t="n">
-        <v>0.1618</v>
-      </c>
-      <c r="BY28" s="3" t="n">
-        <v>0.0882</v>
-      </c>
-      <c r="BZ28" s="3" t="n">
-        <v>0.2353</v>
-      </c>
-      <c r="CA28" s="3" t="n">
-        <v>0.0294</v>
-      </c>
-      <c r="CB28" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="CC28" s="3" t="n">
-        <v>7.66</v>
-      </c>
-      <c r="CD28" s="3" t="n">
-        <v>2</v>
-      </c>
       <c r="CE28" s="3" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CF28" s="3" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="CG28" s="3" t="n">
-        <v>0.096</v>
+        <v>0.1787</v>
       </c>
       <c r="CH28" s="3" t="n">
-        <v>0.0396</v>
+        <v>0.0711</v>
       </c>
       <c r="CI28" s="3" t="n">
-        <v>0.0033</v>
+        <v>0.0042</v>
       </c>
       <c r="CJ28" s="3" t="n">
-        <v>0.0369</v>
+        <v>0.0405</v>
       </c>
       <c r="CK28" s="3" t="n">
-        <v>0.1029</v>
+        <v>0.1064</v>
       </c>
       <c r="CL28" s="3" t="n">
-        <v>0.0065</v>
+        <v>0.0109</v>
       </c>
       <c r="CM28" s="3" t="n">
-        <v>0.1514</v>
+        <v>0.1268</v>
       </c>
       <c r="CN28" s="3" t="n">
-        <v>0.1071</v>
+        <v>0.1325</v>
       </c>
       <c r="CO28" s="3" t="n">
-        <v>0.019</v>
+        <v>0.0092</v>
       </c>
       <c r="CP28" s="4" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -9525,22 +9525,22 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Elly De La Cruz</t>
+          <t>James Wood</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>CIN</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>NYY</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>CHC @ CIN</t>
+          <t>NYY @ WSH</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
@@ -9550,62 +9550,62 @@
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>RF</t>
         </is>
       </c>
       <c r="J29" s="3" t="n">
-        <v>9.77</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>9.56</v>
+        <v>7.94</v>
       </c>
       <c r="L29" s="5" t="n">
-        <v>78.5</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="M29" s="5" t="n">
-        <v>69.5</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="N29" s="5" t="n">
-        <v>69.5</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="O29" s="5" t="n">
-        <v>66.2</v>
+        <v>59.5</v>
       </c>
       <c r="P29" s="5" t="n">
-        <v>66.2</v>
+        <v>59.5</v>
       </c>
       <c r="Q29" s="6" t="n">
-        <v>56.3</v>
+        <v>49.2</v>
       </c>
       <c r="R29" s="7" t="n">
-        <v>56.3</v>
+        <v>49.2</v>
       </c>
       <c r="S29" s="7" t="n">
-        <v>53</v>
+        <v>45.8</v>
       </c>
       <c r="T29" s="7" t="n">
-        <v>53</v>
-      </c>
-      <c r="U29" s="7" t="n">
-        <v>47.2</v>
-      </c>
-      <c r="V29" s="7" t="n">
-        <v>47.2</v>
-      </c>
-      <c r="W29" s="7" t="n">
-        <v>43.1</v>
-      </c>
-      <c r="X29" s="7" t="n">
-        <v>43.1</v>
-      </c>
-      <c r="Y29" s="7" t="n">
-        <v>40.2</v>
-      </c>
-      <c r="Z29" s="7" t="n">
-        <v>40.2</v>
+        <v>45.8</v>
+      </c>
+      <c r="U29" s="9" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="V29" s="9" t="n">
+        <v>38.6</v>
+      </c>
+      <c r="W29" s="9" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="X29" s="9" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="Y29" s="9" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="Z29" s="9" t="n">
+        <v>31.3</v>
       </c>
       <c r="AA29" s="3" t="n">
-        <v>234.73</v>
+        <v>234.68</v>
       </c>
       <c r="AB29" s="4" t="inlineStr">
         <is>
@@ -9614,14 +9614,14 @@
       </c>
       <c r="AC29" s="8" t="inlineStr">
         <is>
-          <t>Forecast 9.8 FS | Sim 9.6</t>
+          <t>Forecast 8.8 FS | Sim 7.9</t>
         </is>
       </c>
       <c r="AD29" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AE29" s="3" t="n">
-        <v>4.84</v>
+        <v>5.13</v>
       </c>
       <c r="AF29" s="4" t="inlineStr">
         <is>
@@ -9636,7 +9636,7 @@
       </c>
       <c r="AI29" s="4" t="inlineStr">
         <is>
-          <t>Javier Assad</t>
+          <t>Cam Schlittler</t>
         </is>
       </c>
       <c r="AJ29" s="4" t="inlineStr">
@@ -9645,179 +9645,179 @@
         </is>
       </c>
       <c r="AK29" s="3" t="n">
-        <v>4.15</v>
+        <v>2.01</v>
       </c>
       <c r="AL29" s="3" t="n">
-        <v>1.1</v>
+        <v>0.93</v>
       </c>
       <c r="AM29" s="3" t="n">
-        <v>0.2098</v>
+        <v>0.1878</v>
       </c>
       <c r="AN29" s="3" t="n">
-        <v>0.0446</v>
+        <v>0.0226</v>
       </c>
       <c r="AO29" s="3" t="n">
-        <v>0.067</v>
+        <v>0.0475</v>
       </c>
       <c r="AP29" s="3" t="n">
-        <v>4.35</v>
+        <v>3.4</v>
       </c>
       <c r="AQ29" s="3" t="n">
-        <v>1.28</v>
+        <v>1.19</v>
       </c>
       <c r="AR29" s="3" t="n">
-        <v>0.2202</v>
+        <v>0.2049</v>
       </c>
       <c r="AS29" s="3" t="n">
-        <v>0.041</v>
+        <v>0.0267</v>
       </c>
       <c r="AT29" s="4" t="inlineStr">
         <is>
-          <t>Great American Ball Park</t>
+          <t>Nationals Park</t>
         </is>
       </c>
       <c r="AU29" s="3" t="n">
-        <v>1.08</v>
+        <v>1</v>
       </c>
       <c r="AV29" s="3" t="n">
-        <v>1.01</v>
+        <v>1.03</v>
       </c>
       <c r="AW29" s="3" t="n">
-        <v>72.90000000000001</v>
+        <v>84.2</v>
       </c>
       <c r="AX29" s="3" t="n">
-        <v>9.699999999999999</v>
+        <v>4.8</v>
       </c>
       <c r="AY29" s="3" t="n">
-        <v>48</v>
+        <v>332</v>
       </c>
       <c r="AZ29" s="3" t="n">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="BA29" s="4" t="inlineStr">
         <is>
-          <t>humid</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="BB29" s="3" t="n">
-        <v>330</v>
+        <v>445</v>
       </c>
       <c r="BC29" s="3" t="n">
-        <v>294</v>
+        <v>362</v>
       </c>
       <c r="BD29" s="3" t="n">
-        <v>0.272</v>
+        <v>0.273</v>
       </c>
       <c r="BE29" s="3" t="n">
-        <v>0.345</v>
+        <v>0.404</v>
       </c>
       <c r="BF29" s="3" t="n">
-        <v>0.497</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="BG29" s="3" t="n">
-        <v>0.842</v>
+        <v>0.962</v>
       </c>
       <c r="BH29" s="3" t="n">
-        <v>231</v>
+        <v>296</v>
       </c>
       <c r="BI29" s="3" t="n">
-        <v>0.738</v>
+        <v>0.997</v>
       </c>
       <c r="BJ29" s="3" t="n">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="BK29" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="BL29" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM29" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="BN29" s="3" t="n">
+        <v>87</v>
+      </c>
+      <c r="BO29" s="3" t="n">
+        <v>62</v>
+      </c>
+      <c r="BP29" s="3" t="n">
+        <v>77</v>
+      </c>
+      <c r="BQ29" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="BR29" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="BL29" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="BM29" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="BN29" s="3" t="n">
-        <v>49</v>
-      </c>
-      <c r="BO29" s="3" t="n">
-        <v>44</v>
-      </c>
-      <c r="BP29" s="3" t="n">
-        <v>32</v>
-      </c>
-      <c r="BQ29" s="3" t="n">
+      <c r="BS29" s="3" t="n">
+        <v>19.14</v>
+      </c>
+      <c r="BT29" s="3" t="n">
+        <v>14.86</v>
+      </c>
+      <c r="BU29" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="BV29" s="3" t="n">
+        <v>3.059</v>
+      </c>
+      <c r="BW29" s="3" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="BX29" s="3" t="n">
+        <v>0.1618</v>
+      </c>
+      <c r="BY29" s="3" t="n">
+        <v>0.0882</v>
+      </c>
+      <c r="BZ29" s="3" t="n">
+        <v>0.2353</v>
+      </c>
+      <c r="CA29" s="3" t="n">
+        <v>0.0294</v>
+      </c>
+      <c r="CB29" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="CC29" s="3" t="n">
+        <v>7.66</v>
+      </c>
+      <c r="CD29" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="BR29" s="3" t="n">
-        <v>13</v>
-      </c>
-      <c r="BS29" s="3" t="n">
-        <v>12.43</v>
-      </c>
-      <c r="BT29" s="3" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="BU29" s="3" t="n">
-        <v>8.57</v>
-      </c>
-      <c r="BV29" s="3" t="n">
-        <v>2.078</v>
-      </c>
-      <c r="BW29" s="3" t="n">
-        <v>0.2188</v>
-      </c>
-      <c r="BX29" s="3" t="n">
-        <v>0.09379999999999999</v>
-      </c>
-      <c r="BY29" s="3" t="n">
-        <v>0.0469</v>
-      </c>
-      <c r="BZ29" s="3" t="n">
-        <v>0.125</v>
-      </c>
-      <c r="CA29" s="3" t="n">
-        <v>0.0469</v>
-      </c>
-      <c r="CB29" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="CC29" s="3" t="n">
-        <v>8.609999999999999</v>
-      </c>
-      <c r="CD29" s="3" t="n">
-        <v>3</v>
-      </c>
       <c r="CE29" s="3" t="n">
-        <v>14.25</v>
+        <v>12</v>
       </c>
       <c r="CF29" s="3" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="CG29" s="3" t="n">
-        <v>0.132</v>
+        <v>0.096</v>
       </c>
       <c r="CH29" s="3" t="n">
-        <v>0.0453</v>
+        <v>0.0396</v>
       </c>
       <c r="CI29" s="3" t="n">
-        <v>0.0062</v>
+        <v>0.0033</v>
       </c>
       <c r="CJ29" s="3" t="n">
-        <v>0.0559</v>
+        <v>0.0369</v>
       </c>
       <c r="CK29" s="3" t="n">
-        <v>0.0813</v>
+        <v>0.1029</v>
       </c>
       <c r="CL29" s="3" t="n">
-        <v>0.0075</v>
+        <v>0.0065</v>
       </c>
       <c r="CM29" s="3" t="n">
-        <v>0.1251</v>
+        <v>0.1514</v>
       </c>
       <c r="CN29" s="3" t="n">
-        <v>0.129</v>
+        <v>0.1071</v>
       </c>
       <c r="CO29" s="3" t="n">
-        <v>0.0206</v>
+        <v>0.019</v>
       </c>
       <c r="CP29" s="4" t="inlineStr">
         <is>
@@ -9839,22 +9839,22 @@
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Trevor Larnach</t>
+          <t>Elly De La Cruz</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>CIN</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>LAA</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>LAA @ MIN</t>
+          <t>CHC @ CIN</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
@@ -9864,62 +9864,62 @@
       </c>
       <c r="I30" s="4" t="inlineStr">
         <is>
-          <t>LF</t>
+          <t>SS</t>
         </is>
       </c>
       <c r="J30" s="3" t="n">
-        <v>9.630000000000001</v>
+        <v>9.77</v>
       </c>
       <c r="K30" s="3" t="n">
-        <v>9.699999999999999</v>
+        <v>9.550000000000001</v>
       </c>
       <c r="L30" s="5" t="n">
-        <v>85.2</v>
+        <v>78.5</v>
       </c>
       <c r="M30" s="5" t="n">
-        <v>76.8</v>
+        <v>69.5</v>
       </c>
       <c r="N30" s="5" t="n">
-        <v>76.8</v>
+        <v>69.5</v>
       </c>
       <c r="O30" s="5" t="n">
-        <v>73.40000000000001</v>
+        <v>66.2</v>
       </c>
       <c r="P30" s="5" t="n">
-        <v>73.40000000000001</v>
-      </c>
-      <c r="Q30" s="5" t="n">
-        <v>62.6</v>
-      </c>
-      <c r="R30" s="5" t="n">
-        <v>62.6</v>
-      </c>
-      <c r="S30" s="5" t="n">
-        <v>58.5</v>
-      </c>
-      <c r="T30" s="5" t="n">
-        <v>58.5</v>
-      </c>
-      <c r="U30" s="6" t="n">
-        <v>50.5</v>
+        <v>66.2</v>
+      </c>
+      <c r="Q30" s="6" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="R30" s="7" t="n">
+        <v>56.2</v>
+      </c>
+      <c r="S30" s="7" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="T30" s="7" t="n">
+        <v>52.9</v>
+      </c>
+      <c r="U30" s="7" t="n">
+        <v>47.2</v>
       </c>
       <c r="V30" s="7" t="n">
-        <v>50.5</v>
+        <v>47.2</v>
       </c>
       <c r="W30" s="7" t="n">
-        <v>44.9</v>
+        <v>43.1</v>
       </c>
       <c r="X30" s="7" t="n">
-        <v>44.9</v>
+        <v>43.1</v>
       </c>
       <c r="Y30" s="7" t="n">
-        <v>41</v>
+        <v>40.2</v>
       </c>
       <c r="Z30" s="7" t="n">
-        <v>41</v>
+        <v>40.2</v>
       </c>
       <c r="AA30" s="3" t="n">
-        <v>234.73</v>
+        <v>234.65</v>
       </c>
       <c r="AB30" s="4" t="inlineStr">
         <is>
@@ -9928,14 +9928,14 @@
       </c>
       <c r="AC30" s="8" t="inlineStr">
         <is>
-          <t>Forecast 9.6 FS | Sim 9.7</t>
+          <t>Forecast 9.8 FS | Sim 9.6</t>
         </is>
       </c>
       <c r="AD30" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AE30" s="3" t="n">
-        <v>4.52</v>
+        <v>4.84</v>
       </c>
       <c r="AF30" s="4" t="inlineStr">
         <is>
@@ -9943,14 +9943,14 @@
         </is>
       </c>
       <c r="AG30" s="3" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AH30" s="3" t="n">
         <v>1.04</v>
       </c>
       <c r="AI30" s="4" t="inlineStr">
         <is>
-          <t>Ryan Johnson</t>
+          <t>Javier Assad</t>
         </is>
       </c>
       <c r="AJ30" s="4" t="inlineStr">
@@ -9959,146 +9959,146 @@
         </is>
       </c>
       <c r="AK30" s="3" t="n">
-        <v>6.99</v>
+        <v>4.15</v>
       </c>
       <c r="AL30" s="3" t="n">
-        <v>1.55</v>
+        <v>1.1</v>
       </c>
       <c r="AM30" s="3" t="n">
-        <v>0.2595</v>
+        <v>0.2098</v>
       </c>
       <c r="AN30" s="3" t="n">
-        <v>0.0611</v>
+        <v>0.0446</v>
       </c>
       <c r="AO30" s="3" t="n">
-        <v>0.07630000000000001</v>
+        <v>0.067</v>
       </c>
       <c r="AP30" s="3" t="n">
-        <v>4.65</v>
+        <v>4.35</v>
       </c>
       <c r="AQ30" s="3" t="n">
-        <v>1.4</v>
+        <v>1.28</v>
       </c>
       <c r="AR30" s="3" t="n">
-        <v>0.2052</v>
+        <v>0.2202</v>
       </c>
       <c r="AS30" s="3" t="n">
-        <v>0.028</v>
+        <v>0.041</v>
       </c>
       <c r="AT30" s="4" t="inlineStr">
         <is>
-          <t>Target Field</t>
+          <t>Great American Ball Park</t>
         </is>
       </c>
       <c r="AU30" s="3" t="n">
-        <v>0.98</v>
+        <v>1.08</v>
       </c>
       <c r="AV30" s="3" t="n">
-        <v>1.03</v>
+        <v>1.01</v>
       </c>
       <c r="AW30" s="3" t="n">
-        <v>88.8</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="AX30" s="3" t="n">
-        <v>5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="AY30" s="3" t="n">
-        <v>188</v>
+        <v>48</v>
       </c>
       <c r="AZ30" s="3" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="BA30" s="4" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>humid</t>
         </is>
       </c>
       <c r="BB30" s="3" t="n">
-        <v>284</v>
+        <v>330</v>
       </c>
       <c r="BC30" s="3" t="n">
-        <v>246</v>
+        <v>294</v>
       </c>
       <c r="BD30" s="3" t="n">
-        <v>0.285</v>
+        <v>0.272</v>
       </c>
       <c r="BE30" s="3" t="n">
-        <v>0.378</v>
+        <v>0.345</v>
       </c>
       <c r="BF30" s="3" t="n">
-        <v>0.439</v>
+        <v>0.497</v>
       </c>
       <c r="BG30" s="3" t="n">
-        <v>0.8169999999999999</v>
+        <v>0.842</v>
       </c>
       <c r="BH30" s="3" t="n">
-        <v>250</v>
+        <v>231</v>
       </c>
       <c r="BI30" s="3" t="n">
-        <v>0.833</v>
+        <v>0.738</v>
       </c>
       <c r="BJ30" s="3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="BK30" s="3" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="BL30" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BM30" s="3" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="BN30" s="3" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="BO30" s="3" t="n">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="BP30" s="3" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="BQ30" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="BR30" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="BS30" s="3" t="n">
+        <v>12.43</v>
+      </c>
+      <c r="BT30" s="3" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="BU30" s="3" t="n">
+        <v>8.57</v>
+      </c>
+      <c r="BV30" s="3" t="n">
+        <v>2.078</v>
+      </c>
+      <c r="BW30" s="3" t="n">
+        <v>0.2188</v>
+      </c>
+      <c r="BX30" s="3" t="n">
+        <v>0.09379999999999999</v>
+      </c>
+      <c r="BY30" s="3" t="n">
+        <v>0.0469</v>
+      </c>
+      <c r="BZ30" s="3" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="CA30" s="3" t="n">
+        <v>0.0469</v>
+      </c>
+      <c r="CB30" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="CC30" s="3" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="CD30" s="3" t="n">
         <v>3</v>
-      </c>
-      <c r="BR30" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="BS30" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="BT30" s="3" t="n">
-        <v>7.07</v>
-      </c>
-      <c r="BU30" s="3" t="n">
-        <v>7.53</v>
-      </c>
-      <c r="BV30" s="3" t="n">
-        <v>1.868</v>
-      </c>
-      <c r="BW30" s="3" t="n">
-        <v>0.2642</v>
-      </c>
-      <c r="BX30" s="3" t="n">
-        <v>0.1321</v>
-      </c>
-      <c r="BY30" s="3" t="n">
-        <v>0.0189</v>
-      </c>
-      <c r="BZ30" s="3" t="n">
-        <v>0.1132</v>
-      </c>
-      <c r="CA30" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB30" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="CC30" s="3" t="n">
-        <v>7.71</v>
-      </c>
-      <c r="CD30" s="3" t="n">
-        <v>4</v>
       </c>
       <c r="CE30" s="3" t="n">
         <v>14</v>
@@ -10107,35 +10107,35 @@
         <v>21</v>
       </c>
       <c r="CG30" s="3" t="n">
-        <v>0.1787</v>
+        <v>0.132</v>
       </c>
       <c r="CH30" s="3" t="n">
-        <v>0.0711</v>
+        <v>0.0453</v>
       </c>
       <c r="CI30" s="3" t="n">
-        <v>0.0042</v>
+        <v>0.0062</v>
       </c>
       <c r="CJ30" s="3" t="n">
-        <v>0.0405</v>
+        <v>0.0559</v>
       </c>
       <c r="CK30" s="3" t="n">
-        <v>0.1064</v>
+        <v>0.0813</v>
       </c>
       <c r="CL30" s="3" t="n">
-        <v>0.0109</v>
+        <v>0.0075</v>
       </c>
       <c r="CM30" s="3" t="n">
-        <v>0.1268</v>
+        <v>0.1251</v>
       </c>
       <c r="CN30" s="3" t="n">
-        <v>0.1325</v>
+        <v>0.129</v>
       </c>
       <c r="CO30" s="3" t="n">
-        <v>0.0092</v>
+        <v>0.0206</v>
       </c>
       <c r="CP30" s="4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -10311,13 +10311,13 @@
         <v>1.03</v>
       </c>
       <c r="AW31" s="3" t="n">
-        <v>88.8</v>
+        <v>88.3</v>
       </c>
       <c r="AX31" s="3" t="n">
-        <v>5</v>
+        <v>5.9</v>
       </c>
       <c r="AY31" s="3" t="n">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="AZ31" s="3" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Update MLB hitter fantasy scores 2026-07-11 (2026-07-10 11:12 PM)
</commit_message>
<xml_diff>
--- a/PRIZEPICKS_HITTER_AI_V3_TOP30_2026_07_11.xlsx
+++ b/PRIZEPICKS_HITTER_AI_V3_TOP30_2026_07_11.xlsx
@@ -1124,58 +1124,58 @@
         </is>
       </c>
       <c r="J2" s="3" t="n">
-        <v>11.8</v>
+        <v>11.79</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>12.41</v>
+        <v>12.33</v>
       </c>
       <c r="L2" s="5" t="n">
         <v>89.2</v>
       </c>
       <c r="M2" s="5" t="n">
-        <v>81.90000000000001</v>
+        <v>81.8</v>
       </c>
       <c r="N2" s="5" t="n">
-        <v>81.90000000000001</v>
+        <v>81.8</v>
       </c>
       <c r="O2" s="5" t="n">
-        <v>80</v>
+        <v>79.8</v>
       </c>
       <c r="P2" s="5" t="n">
-        <v>80</v>
+        <v>79.8</v>
       </c>
       <c r="Q2" s="5" t="n">
-        <v>71.2</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="R2" s="5" t="n">
-        <v>71.2</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="S2" s="5" t="n">
-        <v>67.59999999999999</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="T2" s="5" t="n">
-        <v>67.59999999999999</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="U2" s="5" t="n">
-        <v>61.9</v>
+        <v>61.8</v>
       </c>
       <c r="V2" s="5" t="n">
-        <v>61.9</v>
+        <v>61.8</v>
       </c>
       <c r="W2" s="6" t="n">
-        <v>57</v>
+        <v>56.6</v>
       </c>
       <c r="X2" s="7" t="n">
-        <v>57</v>
+        <v>56.6</v>
       </c>
       <c r="Y2" s="7" t="n">
-        <v>54.1</v>
+        <v>53.6</v>
       </c>
       <c r="Z2" s="7" t="n">
-        <v>54.1</v>
+        <v>53.6</v>
       </c>
       <c r="AA2" s="3" t="n">
-        <v>294.94</v>
+        <v>294.69</v>
       </c>
       <c r="AB2" s="4" t="inlineStr">
         <is>
@@ -1184,7 +1184,7 @@
       </c>
       <c r="AC2" s="8" t="inlineStr">
         <is>
-          <t>Forecast 11.8 FS | Sim 12.4</t>
+          <t>Forecast 11.8 FS | Sim 12.3</t>
         </is>
       </c>
       <c r="AD2" s="3" t="n">
@@ -1230,13 +1230,13 @@
         <v>0.0476</v>
       </c>
       <c r="AP2" s="3" t="n">
-        <v>5.46</v>
+        <v>5.47</v>
       </c>
       <c r="AQ2" s="3" t="n">
         <v>1.52</v>
       </c>
       <c r="AR2" s="3" t="n">
-        <v>0.2557</v>
+        <v>0.2555</v>
       </c>
       <c r="AS2" s="3" t="n">
         <v>0.0346</v>
@@ -1270,7 +1270,7 @@
         </is>
       </c>
       <c r="BB2" s="3" t="n">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="BC2" s="3" t="n">
         <v>359</v>
@@ -1279,13 +1279,13 @@
         <v>0.253</v>
       </c>
       <c r="BE2" s="3" t="n">
-        <v>0.322</v>
+        <v>0.321</v>
       </c>
       <c r="BF2" s="3" t="n">
         <v>0.487</v>
       </c>
       <c r="BG2" s="3" t="n">
-        <v>0.8090000000000001</v>
+        <v>0.8080000000000001</v>
       </c>
       <c r="BH2" s="3" t="n">
         <v>131</v>
@@ -1309,7 +1309,7 @@
         <v>48</v>
       </c>
       <c r="BO2" s="3" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="BP2" s="3" t="n">
         <v>36</v>
@@ -1321,28 +1321,28 @@
         <v>0</v>
       </c>
       <c r="BS2" s="3" t="n">
-        <v>12.57</v>
+        <v>12.86</v>
       </c>
       <c r="BT2" s="3" t="n">
-        <v>12.5</v>
+        <v>12.64</v>
       </c>
       <c r="BU2" s="3" t="n">
-        <v>10.07</v>
+        <v>10.13</v>
       </c>
       <c r="BV2" s="3" t="n">
-        <v>3.017</v>
+        <v>3</v>
       </c>
       <c r="BW2" s="3" t="n">
-        <v>0.3103</v>
+        <v>0.3051</v>
       </c>
       <c r="BX2" s="3" t="n">
-        <v>0.1552</v>
+        <v>0.1525</v>
       </c>
       <c r="BY2" s="3" t="n">
-        <v>0.1207</v>
+        <v>0.1186</v>
       </c>
       <c r="BZ2" s="3" t="n">
-        <v>0.1552</v>
+        <v>0.1525</v>
       </c>
       <c r="CA2" s="3" t="n">
         <v>0</v>
@@ -1351,40 +1351,40 @@
         <v>10</v>
       </c>
       <c r="CC2" s="3" t="n">
-        <v>9.33</v>
+        <v>9.26</v>
       </c>
       <c r="CD2" s="3" t="n">
         <v>5</v>
       </c>
       <c r="CE2" s="3" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="CF2" s="3" t="n">
         <v>26</v>
       </c>
       <c r="CG2" s="3" t="n">
-        <v>0.1905</v>
+        <v>0.19</v>
       </c>
       <c r="CH2" s="3" t="n">
-        <v>0.0654</v>
+        <v>0.0653</v>
       </c>
       <c r="CI2" s="3" t="n">
         <v>0.0043</v>
       </c>
       <c r="CJ2" s="3" t="n">
-        <v>0.0646</v>
+        <v>0.0644</v>
       </c>
       <c r="CK2" s="3" t="n">
-        <v>0.0674</v>
+        <v>0.0673</v>
       </c>
       <c r="CL2" s="3" t="n">
         <v>0.0056</v>
       </c>
       <c r="CM2" s="3" t="n">
-        <v>0.1495</v>
+        <v>0.149</v>
       </c>
       <c r="CN2" s="3" t="n">
-        <v>0.1203</v>
+        <v>0.1223</v>
       </c>
       <c r="CO2" s="3" t="n">
         <v>0.0075</v>
@@ -1441,55 +1441,55 @@
         <v>11.65</v>
       </c>
       <c r="K3" s="3" t="n">
-        <v>11.75</v>
+        <v>11.76</v>
       </c>
       <c r="L3" s="5" t="n">
-        <v>84.59999999999999</v>
+        <v>84.7</v>
       </c>
       <c r="M3" s="5" t="n">
-        <v>77</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="N3" s="5" t="n">
-        <v>77</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="O3" s="5" t="n">
-        <v>73.8</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="P3" s="5" t="n">
-        <v>73.8</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="Q3" s="5" t="n">
-        <v>64.8</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="R3" s="5" t="n">
-        <v>64.8</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="S3" s="5" t="n">
-        <v>61.7</v>
+        <v>61.8</v>
       </c>
       <c r="T3" s="5" t="n">
-        <v>61.7</v>
+        <v>61.8</v>
       </c>
       <c r="U3" s="6" t="n">
-        <v>56.1</v>
+        <v>56.2</v>
       </c>
       <c r="V3" s="7" t="n">
-        <v>56.1</v>
+        <v>56.2</v>
       </c>
       <c r="W3" s="7" t="n">
-        <v>52.1</v>
+        <v>52.2</v>
       </c>
       <c r="X3" s="7" t="n">
-        <v>52.1</v>
+        <v>52.2</v>
       </c>
       <c r="Y3" s="7" t="n">
-        <v>49.1</v>
+        <v>49.2</v>
       </c>
       <c r="Z3" s="7" t="n">
-        <v>49.1</v>
+        <v>49.2</v>
       </c>
       <c r="AA3" s="3" t="n">
-        <v>277.27</v>
+        <v>277.38</v>
       </c>
       <c r="AB3" s="4" t="inlineStr">
         <is>
@@ -1576,7 +1576,7 @@
         <v>332</v>
       </c>
       <c r="AZ3" s="3" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="BA3" s="4" t="inlineStr">
         <is>
@@ -1755,7 +1755,7 @@
         <v>10.96</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>10.65</v>
+        <v>10.66</v>
       </c>
       <c r="L4" s="5" t="n">
         <v>85</v>
@@ -1773,10 +1773,10 @@
         <v>74</v>
       </c>
       <c r="Q4" s="5" t="n">
-        <v>65.2</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="R4" s="5" t="n">
-        <v>65.2</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="S4" s="5" t="n">
         <v>61.4</v>
@@ -1797,13 +1797,13 @@
         <v>49.9</v>
       </c>
       <c r="Y4" s="7" t="n">
-        <v>45.7</v>
+        <v>45.8</v>
       </c>
       <c r="Z4" s="7" t="n">
-        <v>45.7</v>
+        <v>45.8</v>
       </c>
       <c r="AA4" s="3" t="n">
-        <v>277.01</v>
+        <v>277.08</v>
       </c>
       <c r="AB4" s="4" t="inlineStr">
         <is>
@@ -1890,7 +1890,7 @@
         <v>48</v>
       </c>
       <c r="AZ4" s="3" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="BA4" s="4" t="inlineStr">
         <is>
@@ -1979,7 +1979,7 @@
         <v>8</v>
       </c>
       <c r="CC4" s="3" t="n">
-        <v>8.390000000000001</v>
+        <v>8.4</v>
       </c>
       <c r="CD4" s="3" t="n">
         <v>4</v>
@@ -2069,10 +2069,10 @@
         <v>11.17</v>
       </c>
       <c r="K5" s="3" t="n">
-        <v>11.48</v>
+        <v>11.5</v>
       </c>
       <c r="L5" s="5" t="n">
-        <v>91.7</v>
+        <v>91.59999999999999</v>
       </c>
       <c r="M5" s="5" t="n">
         <v>83</v>
@@ -2093,10 +2093,10 @@
         <v>73.5</v>
       </c>
       <c r="S5" s="5" t="n">
-        <v>68.5</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="T5" s="5" t="n">
-        <v>68.5</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="U5" s="5" t="n">
         <v>63.8</v>
@@ -2117,7 +2117,7 @@
         <v>53.2</v>
       </c>
       <c r="AA5" s="3" t="n">
-        <v>273.31</v>
+        <v>273.46</v>
       </c>
       <c r="AB5" s="4" t="inlineStr">
         <is>
@@ -2172,13 +2172,13 @@
         <v>0.0476</v>
       </c>
       <c r="AP5" s="3" t="n">
-        <v>5.46</v>
+        <v>5.47</v>
       </c>
       <c r="AQ5" s="3" t="n">
         <v>1.52</v>
       </c>
       <c r="AR5" s="3" t="n">
-        <v>0.2557</v>
+        <v>0.2555</v>
       </c>
       <c r="AS5" s="3" t="n">
         <v>0.0346</v>
@@ -2293,7 +2293,7 @@
         <v>10</v>
       </c>
       <c r="CC5" s="3" t="n">
-        <v>8.02</v>
+        <v>8.06</v>
       </c>
       <c r="CD5" s="3" t="n">
         <v>5</v>
@@ -2305,7 +2305,7 @@
         <v>23</v>
       </c>
       <c r="CG5" s="3" t="n">
-        <v>0.2607</v>
+        <v>0.2606</v>
       </c>
       <c r="CH5" s="3" t="n">
         <v>0.07099999999999999</v>
@@ -2317,7 +2317,7 @@
         <v>0.0307</v>
       </c>
       <c r="CK5" s="3" t="n">
-        <v>0.0499</v>
+        <v>0.05</v>
       </c>
       <c r="CL5" s="3" t="n">
         <v>0.0068</v>
@@ -3014,7 +3014,7 @@
         <v>11.52</v>
       </c>
       <c r="L8" s="5" t="n">
-        <v>85.7</v>
+        <v>85.8</v>
       </c>
       <c r="M8" s="5" t="n">
         <v>79.7</v>
@@ -3023,10 +3023,10 @@
         <v>79.7</v>
       </c>
       <c r="O8" s="5" t="n">
-        <v>76.5</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="P8" s="5" t="n">
-        <v>76.5</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="Q8" s="5" t="n">
         <v>67.3</v>
@@ -3331,16 +3331,16 @@
         <v>82.90000000000001</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>76.09999999999999</v>
+        <v>76.2</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>76.09999999999999</v>
+        <v>76.2</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>72.09999999999999</v>
+        <v>72.2</v>
       </c>
       <c r="P9" s="5" t="n">
-        <v>72.09999999999999</v>
+        <v>72.2</v>
       </c>
       <c r="Q9" s="5" t="n">
         <v>62.8</v>
@@ -3555,7 +3555,7 @@
         <v>4</v>
       </c>
       <c r="CE9" s="3" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="CF9" s="3" t="n">
         <v>23</v>
@@ -3953,7 +3953,7 @@
         <v>10.17</v>
       </c>
       <c r="K11" s="3" t="n">
-        <v>10.48</v>
+        <v>10.47</v>
       </c>
       <c r="L11" s="5" t="n">
         <v>87.5</v>
@@ -3971,28 +3971,28 @@
         <v>76.8</v>
       </c>
       <c r="Q11" s="5" t="n">
-        <v>67.40000000000001</v>
+        <v>67.3</v>
       </c>
       <c r="R11" s="5" t="n">
-        <v>67.40000000000001</v>
+        <v>67.3</v>
       </c>
       <c r="S11" s="5" t="n">
-        <v>62.9</v>
+        <v>62.8</v>
       </c>
       <c r="T11" s="5" t="n">
-        <v>62.9</v>
+        <v>62.8</v>
       </c>
       <c r="U11" s="6" t="n">
-        <v>55.9</v>
+        <v>55.8</v>
       </c>
       <c r="V11" s="7" t="n">
-        <v>55.9</v>
+        <v>55.8</v>
       </c>
       <c r="W11" s="7" t="n">
-        <v>49.9</v>
+        <v>49.8</v>
       </c>
       <c r="X11" s="7" t="n">
-        <v>49.9</v>
+        <v>49.8</v>
       </c>
       <c r="Y11" s="7" t="n">
         <v>45.3</v>
@@ -4001,7 +4001,7 @@
         <v>45.3</v>
       </c>
       <c r="AA11" s="3" t="n">
-        <v>251.56</v>
+        <v>251.46</v>
       </c>
       <c r="AB11" s="4" t="inlineStr">
         <is>
@@ -4235,22 +4235,22 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Shohei Ohtani</t>
+          <t>Casey Schmitt</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>LAD</t>
+          <t>SF</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>ARI</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>ARI @ LAD</t>
+          <t>COL @ SF</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -4260,62 +4260,62 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>TWP</t>
+          <t>LF</t>
         </is>
       </c>
       <c r="J12" s="3" t="n">
-        <v>10.32</v>
+        <v>10.96</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>10.19</v>
+        <v>10.98</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>82.90000000000001</v>
+        <v>88.59999999999999</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>75.59999999999999</v>
+        <v>78.2</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>75.59999999999999</v>
+        <v>78.2</v>
       </c>
       <c r="O12" s="5" t="n">
-        <v>70.7</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="P12" s="5" t="n">
-        <v>70.7</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="Q12" s="5" t="n">
-        <v>61.8</v>
+        <v>67.8</v>
       </c>
       <c r="R12" s="5" t="n">
-        <v>61.8</v>
-      </c>
-      <c r="S12" s="6" t="n">
-        <v>57.8</v>
-      </c>
-      <c r="T12" s="7" t="n">
-        <v>57.8</v>
-      </c>
-      <c r="U12" s="7" t="n">
-        <v>50.8</v>
+        <v>67.8</v>
+      </c>
+      <c r="S12" s="5" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="T12" s="5" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="U12" s="6" t="n">
+        <v>57.5</v>
       </c>
       <c r="V12" s="7" t="n">
-        <v>50.8</v>
+        <v>57.5</v>
       </c>
       <c r="W12" s="7" t="n">
-        <v>46.3</v>
+        <v>50.6</v>
       </c>
       <c r="X12" s="7" t="n">
-        <v>46.3</v>
+        <v>50.6</v>
       </c>
       <c r="Y12" s="7" t="n">
-        <v>42.6</v>
+        <v>48.4</v>
       </c>
       <c r="Z12" s="7" t="n">
-        <v>42.6</v>
+        <v>48.4</v>
       </c>
       <c r="AA12" s="3" t="n">
-        <v>250.13</v>
+        <v>251.04</v>
       </c>
       <c r="AB12" s="4" t="inlineStr">
         <is>
@@ -4324,14 +4324,14 @@
       </c>
       <c r="AC12" s="8" t="inlineStr">
         <is>
-          <t>Forecast 10.3 FS | Sim 10.2</t>
+          <t>Forecast 11.0 FS | Sim 11.0</t>
         </is>
       </c>
       <c r="AD12" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AE12" s="3" t="n">
-        <v>4.92</v>
+        <v>4.82</v>
       </c>
       <c r="AF12" s="4" t="inlineStr">
         <is>
@@ -4339,191 +4339,199 @@
         </is>
       </c>
       <c r="AG12" s="3" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AH12" s="3" t="n">
         <v>1.04</v>
       </c>
       <c r="AI12" s="4" t="inlineStr">
         <is>
-          <t>Brandon Pfaadt</t>
+          <t>Kyle Freeland</t>
         </is>
       </c>
       <c r="AJ12" s="4" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>L</t>
         </is>
       </c>
       <c r="AK12" s="3" t="n">
-        <v>4.84</v>
+        <v>7.46</v>
       </c>
       <c r="AL12" s="3" t="n">
-        <v>1.34</v>
+        <v>1.61</v>
       </c>
       <c r="AM12" s="3" t="n">
-        <v>0.2249</v>
+        <v>0.3016</v>
       </c>
       <c r="AN12" s="3" t="n">
-        <v>0.0383</v>
+        <v>0.045</v>
       </c>
       <c r="AO12" s="3" t="n">
-        <v>0.0861</v>
+        <v>0.0476</v>
       </c>
       <c r="AP12" s="3" t="n">
-        <v>4.25</v>
+        <v>5.47</v>
       </c>
       <c r="AQ12" s="3" t="n">
-        <v>1.28</v>
+        <v>1.52</v>
       </c>
       <c r="AR12" s="3" t="n">
-        <v>0.2262</v>
+        <v>0.2555</v>
       </c>
       <c r="AS12" s="3" t="n">
-        <v>0.0328</v>
+        <v>0.0346</v>
       </c>
       <c r="AT12" s="4" t="inlineStr">
         <is>
-          <t>UNIQLO Field at Dodger Stadium</t>
+          <t>Oracle Park</t>
         </is>
       </c>
       <c r="AU12" s="3" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="AV12" s="3" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="AW12" s="3" t="n">
+        <v>72.3</v>
+      </c>
+      <c r="AX12" s="3" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="AY12" s="3" t="n">
+        <v>275</v>
+      </c>
+      <c r="AZ12" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="AV12" s="3" t="n">
+      <c r="BA12" s="4" t="inlineStr">
+        <is>
+          <t>light wind</t>
+        </is>
+      </c>
+      <c r="BB12" s="3" t="n">
+        <v>362</v>
+      </c>
+      <c r="BC12" s="3" t="n">
+        <v>342</v>
+      </c>
+      <c r="BD12" s="3" t="n">
+        <v>0.281</v>
+      </c>
+      <c r="BE12" s="3" t="n">
+        <v>0.309</v>
+      </c>
+      <c r="BF12" s="3" t="n">
+        <v>0.494</v>
+      </c>
+      <c r="BG12" s="3" t="n">
+        <v>0.803</v>
+      </c>
+      <c r="BH12" s="3" t="n">
+        <v>97</v>
+      </c>
+      <c r="BI12" s="3" t="n">
+        <v>0.829</v>
+      </c>
+      <c r="BJ12" s="3" t="n">
+        <v>96</v>
+      </c>
+      <c r="BK12" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="BL12" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="AW12" s="4" t="n"/>
-      <c r="AX12" s="4" t="n"/>
-      <c r="AY12" s="4" t="n"/>
-      <c r="AZ12" s="4" t="n"/>
-      <c r="BA12" s="4" t="inlineStr">
-        <is>
-          <t>Weather unavailable</t>
-        </is>
-      </c>
-      <c r="BB12" s="3" t="n">
-        <v>399</v>
-      </c>
-      <c r="BC12" s="3" t="n">
-        <v>328</v>
-      </c>
-      <c r="BD12" s="3" t="n">
-        <v>0.29</v>
-      </c>
-      <c r="BE12" s="3" t="n">
-        <v>0.403</v>
-      </c>
-      <c r="BF12" s="3" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="BG12" s="3" t="n">
-        <v>0.9429999999999999</v>
-      </c>
-      <c r="BH12" s="3" t="n">
-        <v>277</v>
-      </c>
-      <c r="BI12" s="3" t="n">
-        <v>0.971</v>
-      </c>
-      <c r="BJ12" s="3" t="n">
-        <v>95</v>
-      </c>
-      <c r="BK12" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="BL12" s="3" t="n">
-        <v>2</v>
-      </c>
       <c r="BM12" s="3" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="BN12" s="3" t="n">
-        <v>63</v>
+        <v>41</v>
       </c>
       <c r="BO12" s="3" t="n">
-        <v>57</v>
+        <v>47</v>
       </c>
       <c r="BP12" s="3" t="n">
-        <v>60</v>
+        <v>9</v>
       </c>
       <c r="BQ12" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="BR12" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="BS12" s="3" t="n">
+        <v>8.859999999999999</v>
+      </c>
+      <c r="BT12" s="3" t="n">
+        <v>5.64</v>
+      </c>
+      <c r="BU12" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="BS12" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="BT12" s="3" t="n">
-        <v>9.140000000000001</v>
-      </c>
-      <c r="BU12" s="3" t="n">
-        <v>10.3</v>
-      </c>
       <c r="BV12" s="3" t="n">
-        <v>2</v>
+        <v>1.386</v>
       </c>
       <c r="BW12" s="3" t="n">
-        <v>0.25</v>
+        <v>0.193</v>
       </c>
       <c r="BX12" s="3" t="n">
-        <v>0.0625</v>
+        <v>0.0702</v>
       </c>
       <c r="BY12" s="3" t="n">
-        <v>0.0625</v>
+        <v>0.0351</v>
       </c>
       <c r="BZ12" s="3" t="n">
-        <v>0.09379999999999999</v>
+        <v>0.0351</v>
       </c>
       <c r="CA12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="CB12" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="CC12" s="3" t="n">
-        <v>8.449999999999999</v>
+        <v>8.44</v>
       </c>
       <c r="CD12" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="CE12" s="3" t="n">
         <v>16</v>
       </c>
       <c r="CF12" s="3" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="CG12" s="3" t="n">
-        <v>0.1524</v>
+        <v>0.2262</v>
       </c>
       <c r="CH12" s="3" t="n">
-        <v>0.0378</v>
+        <v>0.0625</v>
       </c>
       <c r="CI12" s="3" t="n">
-        <v>0.0043</v>
+        <v>0.0044</v>
       </c>
       <c r="CJ12" s="3" t="n">
-        <v>0.0538</v>
+        <v>0.0526</v>
       </c>
       <c r="CK12" s="3" t="n">
-        <v>0.1184</v>
+        <v>0.0387</v>
       </c>
       <c r="CL12" s="3" t="n">
-        <v>0.0097</v>
+        <v>0.009599999999999999</v>
       </c>
       <c r="CM12" s="3" t="n">
-        <v>0.1327</v>
+        <v>0.126</v>
       </c>
       <c r="CN12" s="3" t="n">
-        <v>0.1522</v>
+        <v>0.1547</v>
       </c>
       <c r="CO12" s="3" t="n">
-        <v>0.0108</v>
+        <v>0.0132</v>
       </c>
       <c r="CP12" s="4" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -4541,22 +4549,22 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Otto Lopez</t>
+          <t>Shohei Ohtani</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>MIA</t>
+          <t>LAD</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>CLE</t>
+          <t>ARI</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>CLE @ MIA</t>
+          <t>ARI @ LAD</t>
         </is>
       </c>
       <c r="H13" s="4" t="inlineStr">
@@ -4566,62 +4574,62 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>TWP</t>
         </is>
       </c>
       <c r="J13" s="3" t="n">
-        <v>9.81</v>
+        <v>10.32</v>
       </c>
       <c r="K13" s="3" t="n">
-        <v>9.539999999999999</v>
+        <v>10.19</v>
       </c>
       <c r="L13" s="5" t="n">
-        <v>82.90000000000001</v>
+        <v>83</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>73.2</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>73.2</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="O13" s="5" t="n">
-        <v>70.59999999999999</v>
+        <v>70.7</v>
       </c>
       <c r="P13" s="5" t="n">
-        <v>70.59999999999999</v>
+        <v>70.7</v>
       </c>
       <c r="Q13" s="5" t="n">
-        <v>60</v>
+        <v>61.8</v>
       </c>
       <c r="R13" s="5" t="n">
-        <v>60</v>
+        <v>61.8</v>
       </c>
       <c r="S13" s="6" t="n">
-        <v>56.6</v>
+        <v>57.8</v>
       </c>
       <c r="T13" s="7" t="n">
-        <v>56.6</v>
+        <v>57.8</v>
       </c>
       <c r="U13" s="7" t="n">
-        <v>50.4</v>
+        <v>50.8</v>
       </c>
       <c r="V13" s="7" t="n">
-        <v>50.4</v>
+        <v>50.8</v>
       </c>
       <c r="W13" s="7" t="n">
-        <v>44.6</v>
+        <v>46.2</v>
       </c>
       <c r="X13" s="7" t="n">
-        <v>44.6</v>
+        <v>46.2</v>
       </c>
       <c r="Y13" s="7" t="n">
-        <v>41.5</v>
+        <v>42.5</v>
       </c>
       <c r="Z13" s="7" t="n">
-        <v>41.5</v>
+        <v>42.5</v>
       </c>
       <c r="AA13" s="3" t="n">
-        <v>249.32</v>
+        <v>250.12</v>
       </c>
       <c r="AB13" s="4" t="inlineStr">
         <is>
@@ -4630,14 +4638,14 @@
       </c>
       <c r="AC13" s="8" t="inlineStr">
         <is>
-          <t>Forecast 9.8 FS | Sim 9.5</t>
+          <t>Forecast 10.3 FS | Sim 10.2</t>
         </is>
       </c>
       <c r="AD13" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AE13" s="3" t="n">
-        <v>5.13</v>
+        <v>4.92</v>
       </c>
       <c r="AF13" s="4" t="inlineStr">
         <is>
@@ -4652,7 +4660,7 @@
       </c>
       <c r="AI13" s="4" t="inlineStr">
         <is>
-          <t>Tanner Bibee</t>
+          <t>Brandon Pfaadt</t>
         </is>
       </c>
       <c r="AJ13" s="4" t="inlineStr">
@@ -4661,39 +4669,39 @@
         </is>
       </c>
       <c r="AK13" s="3" t="n">
-        <v>4.06</v>
+        <v>4.84</v>
       </c>
       <c r="AL13" s="3" t="n">
-        <v>1.14</v>
+        <v>1.34</v>
       </c>
       <c r="AM13" s="3" t="n">
-        <v>0.2116</v>
+        <v>0.2249</v>
       </c>
       <c r="AN13" s="3" t="n">
-        <v>0.0465</v>
+        <v>0.0383</v>
       </c>
       <c r="AO13" s="3" t="n">
-        <v>0.0698</v>
+        <v>0.0861</v>
       </c>
       <c r="AP13" s="3" t="n">
-        <v>3.76</v>
+        <v>4.25</v>
       </c>
       <c r="AQ13" s="3" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AR13" s="3" t="n">
-        <v>0.211</v>
+        <v>0.2262</v>
       </c>
       <c r="AS13" s="3" t="n">
-        <v>0.0308</v>
+        <v>0.0328</v>
       </c>
       <c r="AT13" s="4" t="inlineStr">
         <is>
-          <t>loanDepot park</t>
+          <t>UNIQLO Field at Dodger Stadium</t>
         </is>
       </c>
       <c r="AU13" s="3" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AV13" s="3" t="n">
         <v>1</v>
@@ -4704,128 +4712,128 @@
       <c r="AZ13" s="4" t="n"/>
       <c r="BA13" s="4" t="inlineStr">
         <is>
-          <t>Indoor/retractable neutral</t>
+          <t>Weather unavailable</t>
         </is>
       </c>
       <c r="BB13" s="3" t="n">
-        <v>401</v>
+        <v>399</v>
       </c>
       <c r="BC13" s="3" t="n">
-        <v>372</v>
+        <v>328</v>
       </c>
       <c r="BD13" s="3" t="n">
-        <v>0.341</v>
+        <v>0.29</v>
       </c>
       <c r="BE13" s="3" t="n">
-        <v>0.374</v>
+        <v>0.403</v>
       </c>
       <c r="BF13" s="3" t="n">
-        <v>0.516</v>
+        <v>0.54</v>
       </c>
       <c r="BG13" s="3" t="n">
-        <v>0.89</v>
+        <v>0.9429999999999999</v>
       </c>
       <c r="BH13" s="3" t="n">
-        <v>309</v>
+        <v>277</v>
       </c>
       <c r="BI13" s="3" t="n">
-        <v>0.835</v>
+        <v>0.971</v>
       </c>
       <c r="BJ13" s="3" t="n">
-        <v>127</v>
+        <v>95</v>
       </c>
       <c r="BK13" s="3" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="BL13" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="BM13" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="BN13" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="BO13" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="BP13" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="BQ13" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="BR13" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="BM13" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="BN13" s="3" t="n">
-        <v>61</v>
-      </c>
-      <c r="BO13" s="3" t="n">
-        <v>45</v>
-      </c>
-      <c r="BP13" s="3" t="n">
-        <v>19</v>
-      </c>
-      <c r="BQ13" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="BR13" s="3" t="n">
-        <v>17</v>
-      </c>
       <c r="BS13" s="3" t="n">
-        <v>14.29</v>
+        <v>10</v>
       </c>
       <c r="BT13" s="3" t="n">
-        <v>12.86</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="BU13" s="3" t="n">
-        <v>11.6</v>
+        <v>10.3</v>
       </c>
       <c r="BV13" s="3" t="n">
-        <v>2.769</v>
+        <v>2</v>
       </c>
       <c r="BW13" s="3" t="n">
-        <v>0.3385</v>
+        <v>0.25</v>
       </c>
       <c r="BX13" s="3" t="n">
-        <v>0.1846</v>
+        <v>0.0625</v>
       </c>
       <c r="BY13" s="3" t="n">
-        <v>0.0615</v>
+        <v>0.0625</v>
       </c>
       <c r="BZ13" s="3" t="n">
-        <v>0.0615</v>
+        <v>0.09379999999999999</v>
       </c>
       <c r="CA13" s="3" t="n">
-        <v>0.0154</v>
+        <v>0</v>
       </c>
       <c r="CB13" s="3" t="n">
         <v>8</v>
       </c>
       <c r="CC13" s="3" t="n">
-        <v>7.91</v>
+        <v>8.470000000000001</v>
       </c>
       <c r="CD13" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="CE13" s="3" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="CF13" s="3" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="CG13" s="3" t="n">
-        <v>0.1641</v>
+        <v>0.1524</v>
       </c>
       <c r="CH13" s="3" t="n">
-        <v>0.0508</v>
+        <v>0.0378</v>
       </c>
       <c r="CI13" s="3" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.0043</v>
       </c>
       <c r="CJ13" s="3" t="n">
-        <v>0.0377</v>
+        <v>0.0538</v>
       </c>
       <c r="CK13" s="3" t="n">
-        <v>0.0594</v>
+        <v>0.1184</v>
       </c>
       <c r="CL13" s="3" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.0097</v>
       </c>
       <c r="CM13" s="3" t="n">
-        <v>0.1377</v>
+        <v>0.1327</v>
       </c>
       <c r="CN13" s="3" t="n">
-        <v>0.1015</v>
+        <v>0.1522</v>
       </c>
       <c r="CO13" s="3" t="n">
-        <v>0.0206</v>
+        <v>0.0108</v>
       </c>
       <c r="CP13" s="4" t="inlineStr">
         <is>
@@ -4847,7 +4855,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Casey Schmitt</t>
+          <t>Willy Adames</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -4872,62 +4880,62 @@
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>LF</t>
+          <t>SS</t>
         </is>
       </c>
       <c r="J14" s="3" t="n">
-        <v>10.92</v>
+        <v>10.47</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>10.91</v>
+        <v>10.59</v>
       </c>
       <c r="L14" s="5" t="n">
-        <v>87.8</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="M14" s="5" t="n">
-        <v>77.59999999999999</v>
+        <v>77</v>
       </c>
       <c r="N14" s="5" t="n">
-        <v>77.59999999999999</v>
+        <v>77</v>
       </c>
       <c r="O14" s="5" t="n">
-        <v>76.3</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="P14" s="5" t="n">
-        <v>76.3</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="Q14" s="5" t="n">
-        <v>66.59999999999999</v>
+        <v>64.8</v>
       </c>
       <c r="R14" s="5" t="n">
-        <v>66.59999999999999</v>
+        <v>64.8</v>
       </c>
       <c r="S14" s="5" t="n">
-        <v>61.7</v>
+        <v>61.1</v>
       </c>
       <c r="T14" s="5" t="n">
-        <v>61.7</v>
+        <v>61.1</v>
       </c>
       <c r="U14" s="6" t="n">
-        <v>57</v>
+        <v>55.1</v>
       </c>
       <c r="V14" s="7" t="n">
-        <v>57</v>
+        <v>55.1</v>
       </c>
       <c r="W14" s="7" t="n">
-        <v>50.2</v>
+        <v>49</v>
       </c>
       <c r="X14" s="7" t="n">
-        <v>50.2</v>
+        <v>49</v>
       </c>
       <c r="Y14" s="7" t="n">
-        <v>47.8</v>
+        <v>45.9</v>
       </c>
       <c r="Z14" s="7" t="n">
-        <v>47.8</v>
+        <v>45.9</v>
       </c>
       <c r="AA14" s="3" t="n">
-        <v>249.28</v>
+        <v>249.62</v>
       </c>
       <c r="AB14" s="4" t="inlineStr">
         <is>
@@ -4936,14 +4944,14 @@
       </c>
       <c r="AC14" s="8" t="inlineStr">
         <is>
-          <t>Forecast 10.9 FS | Sim 10.9</t>
+          <t>Forecast 10.5 FS | Sim 10.6</t>
         </is>
       </c>
       <c r="AD14" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AE14" s="3" t="n">
-        <v>4.82</v>
+        <v>4.92</v>
       </c>
       <c r="AF14" s="4" t="inlineStr">
         <is>
@@ -4951,7 +4959,7 @@
         </is>
       </c>
       <c r="AG14" s="3" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="AH14" s="3" t="n">
         <v>1.04</v>
@@ -4982,13 +4990,13 @@
         <v>0.0476</v>
       </c>
       <c r="AP14" s="3" t="n">
-        <v>5.46</v>
+        <v>5.47</v>
       </c>
       <c r="AQ14" s="3" t="n">
         <v>1.52</v>
       </c>
       <c r="AR14" s="3" t="n">
-        <v>0.2557</v>
+        <v>0.2555</v>
       </c>
       <c r="AS14" s="3" t="n">
         <v>0.0346</v>
@@ -5022,88 +5030,88 @@
         </is>
       </c>
       <c r="BB14" s="3" t="n">
-        <v>362</v>
+        <v>376</v>
       </c>
       <c r="BC14" s="3" t="n">
-        <v>342</v>
+        <v>349</v>
       </c>
       <c r="BD14" s="3" t="n">
-        <v>0.278</v>
+        <v>0.226</v>
       </c>
       <c r="BE14" s="3" t="n">
-        <v>0.307</v>
+        <v>0.279</v>
       </c>
       <c r="BF14" s="3" t="n">
-        <v>0.491</v>
+        <v>0.421</v>
       </c>
       <c r="BG14" s="3" t="n">
-        <v>0.798</v>
+        <v>0.7</v>
       </c>
       <c r="BH14" s="3" t="n">
         <v>97</v>
       </c>
       <c r="BI14" s="3" t="n">
-        <v>0.829</v>
+        <v>0.607</v>
       </c>
       <c r="BJ14" s="3" t="n">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="BK14" s="3" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="BL14" s="3" t="n">
         <v>1</v>
       </c>
       <c r="BM14" s="3" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="BN14" s="3" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="BO14" s="3" t="n">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="BP14" s="3" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="BQ14" s="3" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="BR14" s="3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="BS14" s="3" t="n">
         <v>8.43</v>
       </c>
       <c r="BT14" s="3" t="n">
-        <v>5.43</v>
+        <v>7.36</v>
       </c>
       <c r="BU14" s="3" t="n">
-        <v>5.9</v>
+        <v>7.13</v>
       </c>
       <c r="BV14" s="3" t="n">
-        <v>1.357</v>
+        <v>1.807</v>
       </c>
       <c r="BW14" s="3" t="n">
-        <v>0.1786</v>
+        <v>0.2105</v>
       </c>
       <c r="BX14" s="3" t="n">
-        <v>0.07140000000000001</v>
+        <v>0.0877</v>
       </c>
       <c r="BY14" s="3" t="n">
-        <v>0.0357</v>
+        <v>0.0351</v>
       </c>
       <c r="BZ14" s="3" t="n">
-        <v>0.0357</v>
+        <v>0.1404</v>
       </c>
       <c r="CA14" s="3" t="n">
-        <v>0</v>
+        <v>0.0175</v>
       </c>
       <c r="CB14" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="CC14" s="3" t="n">
-        <v>8.550000000000001</v>
+        <v>8.41</v>
       </c>
       <c r="CD14" s="3" t="n">
         <v>5</v>
@@ -5112,34 +5120,34 @@
         <v>16</v>
       </c>
       <c r="CF14" s="3" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="CG14" s="3" t="n">
-        <v>0.2228</v>
+        <v>0.1794</v>
       </c>
       <c r="CH14" s="3" t="n">
-        <v>0.0626</v>
+        <v>0.0664</v>
       </c>
       <c r="CI14" s="3" t="n">
-        <v>0.0044</v>
+        <v>0.005</v>
       </c>
       <c r="CJ14" s="3" t="n">
-        <v>0.0526</v>
+        <v>0.0506</v>
       </c>
       <c r="CK14" s="3" t="n">
-        <v>0.0387</v>
+        <v>0.0604</v>
       </c>
       <c r="CL14" s="3" t="n">
-        <v>0.009599999999999999</v>
+        <v>0.0054</v>
       </c>
       <c r="CM14" s="3" t="n">
-        <v>0.1262</v>
+        <v>0.1384</v>
       </c>
       <c r="CN14" s="3" t="n">
-        <v>0.1549</v>
+        <v>0.1265</v>
       </c>
       <c r="CO14" s="3" t="n">
-        <v>0.0132</v>
+        <v>0.0104</v>
       </c>
       <c r="CP14" s="4" t="inlineStr">
         <is>
@@ -5161,22 +5169,22 @@
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Sal Stewart</t>
+          <t>Otto Lopez</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>CIN</t>
+          <t>MIA</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>CHC</t>
+          <t>CLE</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>CHC @ CIN</t>
+          <t>CLE @ MIA</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
@@ -5186,41 +5194,41 @@
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>1B</t>
+          <t>SS</t>
         </is>
       </c>
       <c r="J15" s="3" t="n">
-        <v>10.47</v>
+        <v>9.81</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>10.42</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="L15" s="5" t="n">
-        <v>80.59999999999999</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="M15" s="5" t="n">
-        <v>72.59999999999999</v>
+        <v>73.2</v>
       </c>
       <c r="N15" s="5" t="n">
-        <v>72.59999999999999</v>
+        <v>73.2</v>
       </c>
       <c r="O15" s="5" t="n">
-        <v>69</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="P15" s="5" t="n">
-        <v>69</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="Q15" s="5" t="n">
-        <v>59.5</v>
+        <v>60.1</v>
       </c>
       <c r="R15" s="5" t="n">
-        <v>59.5</v>
+        <v>60.1</v>
       </c>
       <c r="S15" s="6" t="n">
-        <v>56.5</v>
+        <v>56.6</v>
       </c>
       <c r="T15" s="7" t="n">
-        <v>56.5</v>
+        <v>56.6</v>
       </c>
       <c r="U15" s="7" t="n">
         <v>50.4</v>
@@ -5229,19 +5237,19 @@
         <v>50.4</v>
       </c>
       <c r="W15" s="7" t="n">
-        <v>46.8</v>
+        <v>44.6</v>
       </c>
       <c r="X15" s="7" t="n">
-        <v>46.8</v>
+        <v>44.6</v>
       </c>
       <c r="Y15" s="7" t="n">
-        <v>43.8</v>
+        <v>41.5</v>
       </c>
       <c r="Z15" s="7" t="n">
-        <v>43.8</v>
+        <v>41.5</v>
       </c>
       <c r="AA15" s="3" t="n">
-        <v>248.96</v>
+        <v>249.32</v>
       </c>
       <c r="AB15" s="4" t="inlineStr">
         <is>
@@ -5250,7 +5258,7 @@
       </c>
       <c r="AC15" s="8" t="inlineStr">
         <is>
-          <t>Forecast 10.5 FS | Sim 10.4</t>
+          <t>Forecast 9.8 FS | Sim 9.5</t>
         </is>
       </c>
       <c r="AD15" s="3" t="n">
@@ -5272,7 +5280,7 @@
       </c>
       <c r="AI15" s="4" t="inlineStr">
         <is>
-          <t>Javier Assad</t>
+          <t>Tanner Bibee</t>
         </is>
       </c>
       <c r="AJ15" s="4" t="inlineStr">
@@ -5281,179 +5289,171 @@
         </is>
       </c>
       <c r="AK15" s="3" t="n">
-        <v>4.15</v>
+        <v>4.06</v>
       </c>
       <c r="AL15" s="3" t="n">
-        <v>1.1</v>
+        <v>1.14</v>
       </c>
       <c r="AM15" s="3" t="n">
-        <v>0.2098</v>
+        <v>0.2116</v>
       </c>
       <c r="AN15" s="3" t="n">
-        <v>0.0446</v>
+        <v>0.0465</v>
       </c>
       <c r="AO15" s="3" t="n">
-        <v>0.067</v>
+        <v>0.0698</v>
       </c>
       <c r="AP15" s="3" t="n">
-        <v>4.35</v>
+        <v>3.76</v>
       </c>
       <c r="AQ15" s="3" t="n">
-        <v>1.28</v>
+        <v>1.26</v>
       </c>
       <c r="AR15" s="3" t="n">
-        <v>0.2202</v>
+        <v>0.211</v>
       </c>
       <c r="AS15" s="3" t="n">
-        <v>0.041</v>
+        <v>0.0308</v>
       </c>
       <c r="AT15" s="4" t="inlineStr">
         <is>
-          <t>Great American Ball Park</t>
+          <t>loanDepot park</t>
         </is>
       </c>
       <c r="AU15" s="3" t="n">
-        <v>1.08</v>
+        <v>0.96</v>
       </c>
       <c r="AV15" s="3" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="AW15" s="3" t="n">
-        <v>72.90000000000001</v>
-      </c>
-      <c r="AX15" s="3" t="n">
-        <v>9.699999999999999</v>
-      </c>
-      <c r="AY15" s="3" t="n">
-        <v>48</v>
-      </c>
-      <c r="AZ15" s="3" t="n">
-        <v>33</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="AW15" s="4" t="n"/>
+      <c r="AX15" s="4" t="n"/>
+      <c r="AY15" s="4" t="n"/>
+      <c r="AZ15" s="4" t="n"/>
       <c r="BA15" s="4" t="inlineStr">
         <is>
-          <t>humid</t>
+          <t>Indoor/retractable neutral</t>
         </is>
       </c>
       <c r="BB15" s="3" t="n">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="BC15" s="3" t="n">
-        <v>354</v>
+        <v>372</v>
       </c>
       <c r="BD15" s="3" t="n">
-        <v>0.257</v>
+        <v>0.341</v>
       </c>
       <c r="BE15" s="3" t="n">
-        <v>0.339</v>
+        <v>0.374</v>
       </c>
       <c r="BF15" s="3" t="n">
-        <v>0.477</v>
+        <v>0.516</v>
       </c>
       <c r="BG15" s="3" t="n">
-        <v>0.8159999999999999</v>
+        <v>0.89</v>
       </c>
       <c r="BH15" s="3" t="n">
-        <v>300</v>
+        <v>309</v>
       </c>
       <c r="BI15" s="3" t="n">
-        <v>0.783</v>
+        <v>0.835</v>
       </c>
       <c r="BJ15" s="3" t="n">
-        <v>91</v>
+        <v>127</v>
       </c>
       <c r="BK15" s="3" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="BL15" s="3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="BM15" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="BN15" s="3" t="n">
+        <v>61</v>
+      </c>
+      <c r="BO15" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="BP15" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="BN15" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="BO15" s="3" t="n">
-        <v>65</v>
-      </c>
-      <c r="BP15" s="3" t="n">
-        <v>45</v>
-      </c>
       <c r="BQ15" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BR15" s="3" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="BS15" s="3" t="n">
-        <v>8.710000000000001</v>
+        <v>14.29</v>
       </c>
       <c r="BT15" s="3" t="n">
-        <v>9.859999999999999</v>
+        <v>12.86</v>
       </c>
       <c r="BU15" s="3" t="n">
-        <v>8.800000000000001</v>
+        <v>11.6</v>
       </c>
       <c r="BV15" s="3" t="n">
-        <v>2.262</v>
+        <v>2.769</v>
       </c>
       <c r="BW15" s="3" t="n">
-        <v>0.2787</v>
+        <v>0.3385</v>
       </c>
       <c r="BX15" s="3" t="n">
-        <v>0.1475</v>
+        <v>0.1846</v>
       </c>
       <c r="BY15" s="3" t="n">
-        <v>0.082</v>
+        <v>0.0615</v>
       </c>
       <c r="BZ15" s="3" t="n">
-        <v>0.0492</v>
+        <v>0.0615</v>
       </c>
       <c r="CA15" s="3" t="n">
-        <v>0</v>
+        <v>0.0154</v>
       </c>
       <c r="CB15" s="3" t="n">
         <v>8</v>
       </c>
       <c r="CC15" s="3" t="n">
-        <v>9.109999999999999</v>
+        <v>7.9</v>
       </c>
       <c r="CD15" s="3" t="n">
         <v>3</v>
       </c>
       <c r="CE15" s="3" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="CF15" s="3" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="CG15" s="3" t="n">
-        <v>0.1258</v>
+        <v>0.1641</v>
       </c>
       <c r="CH15" s="3" t="n">
-        <v>0.0526</v>
+        <v>0.0508</v>
       </c>
       <c r="CI15" s="3" t="n">
-        <v>0.0025</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="CJ15" s="3" t="n">
-        <v>0.0649</v>
+        <v>0.0377</v>
       </c>
       <c r="CK15" s="3" t="n">
-        <v>0.079</v>
+        <v>0.0594</v>
       </c>
       <c r="CL15" s="3" t="n">
-        <v>0.0061</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="CM15" s="3" t="n">
-        <v>0.1217</v>
+        <v>0.1377</v>
       </c>
       <c r="CN15" s="3" t="n">
-        <v>0.1243</v>
+        <v>0.1015</v>
       </c>
       <c r="CO15" s="3" t="n">
-        <v>0.0142</v>
+        <v>0.0206</v>
       </c>
       <c r="CP15" s="4" t="inlineStr">
         <is>
@@ -5475,22 +5475,22 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Willy Adames</t>
+          <t>Sal Stewart</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>SF</t>
+          <t>CIN</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>CHC</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>COL @ SF</t>
+          <t>CHC @ CIN</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
@@ -5500,62 +5500,62 @@
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>1B</t>
         </is>
       </c>
       <c r="J16" s="3" t="n">
-        <v>10.48</v>
+        <v>10.47</v>
       </c>
       <c r="K16" s="3" t="n">
-        <v>10.54</v>
+        <v>10.42</v>
       </c>
       <c r="L16" s="5" t="n">
-        <v>85.90000000000001</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="M16" s="5" t="n">
-        <v>76.7</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>76.7</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="O16" s="5" t="n">
-        <v>74.90000000000001</v>
+        <v>69</v>
       </c>
       <c r="P16" s="5" t="n">
-        <v>74.90000000000001</v>
+        <v>69</v>
       </c>
       <c r="Q16" s="5" t="n">
-        <v>64.5</v>
+        <v>59.4</v>
       </c>
       <c r="R16" s="5" t="n">
-        <v>64.5</v>
-      </c>
-      <c r="S16" s="5" t="n">
-        <v>60.7</v>
-      </c>
-      <c r="T16" s="5" t="n">
-        <v>60.7</v>
-      </c>
-      <c r="U16" s="6" t="n">
-        <v>55</v>
+        <v>59.4</v>
+      </c>
+      <c r="S16" s="6" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="T16" s="7" t="n">
+        <v>56.4</v>
+      </c>
+      <c r="U16" s="7" t="n">
+        <v>50.3</v>
       </c>
       <c r="V16" s="7" t="n">
-        <v>55</v>
+        <v>50.3</v>
       </c>
       <c r="W16" s="7" t="n">
-        <v>49</v>
+        <v>46.7</v>
       </c>
       <c r="X16" s="7" t="n">
-        <v>49</v>
+        <v>46.7</v>
       </c>
       <c r="Y16" s="7" t="n">
-        <v>45.9</v>
+        <v>43.8</v>
       </c>
       <c r="Z16" s="7" t="n">
-        <v>45.9</v>
+        <v>43.8</v>
       </c>
       <c r="AA16" s="3" t="n">
-        <v>248.75</v>
+        <v>248.92</v>
       </c>
       <c r="AB16" s="4" t="inlineStr">
         <is>
@@ -5564,14 +5564,14 @@
       </c>
       <c r="AC16" s="8" t="inlineStr">
         <is>
-          <t>Forecast 10.5 FS | Sim 10.5</t>
+          <t>Forecast 10.5 FS | Sim 10.4</t>
         </is>
       </c>
       <c r="AD16" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AE16" s="3" t="n">
-        <v>4.92</v>
+        <v>5.13</v>
       </c>
       <c r="AF16" s="4" t="inlineStr">
         <is>
@@ -5586,192 +5586,192 @@
       </c>
       <c r="AI16" s="4" t="inlineStr">
         <is>
-          <t>Kyle Freeland</t>
+          <t>Javier Assad</t>
         </is>
       </c>
       <c r="AJ16" s="4" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>R</t>
         </is>
       </c>
       <c r="AK16" s="3" t="n">
-        <v>7.46</v>
+        <v>4.15</v>
       </c>
       <c r="AL16" s="3" t="n">
-        <v>1.61</v>
+        <v>1.1</v>
       </c>
       <c r="AM16" s="3" t="n">
-        <v>0.3016</v>
+        <v>0.2098</v>
       </c>
       <c r="AN16" s="3" t="n">
-        <v>0.045</v>
+        <v>0.0446</v>
       </c>
       <c r="AO16" s="3" t="n">
-        <v>0.0476</v>
+        <v>0.067</v>
       </c>
       <c r="AP16" s="3" t="n">
-        <v>5.46</v>
+        <v>4.35</v>
       </c>
       <c r="AQ16" s="3" t="n">
-        <v>1.52</v>
+        <v>1.28</v>
       </c>
       <c r="AR16" s="3" t="n">
-        <v>0.2557</v>
+        <v>0.2202</v>
       </c>
       <c r="AS16" s="3" t="n">
-        <v>0.0346</v>
+        <v>0.041</v>
       </c>
       <c r="AT16" s="4" t="inlineStr">
         <is>
-          <t>Oracle Park</t>
+          <t>Great American Ball Park</t>
         </is>
       </c>
       <c r="AU16" s="3" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.08</v>
       </c>
       <c r="AV16" s="3" t="n">
         <v>1.01</v>
       </c>
       <c r="AW16" s="3" t="n">
-        <v>72.3</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="AX16" s="3" t="n">
-        <v>11.2</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="AY16" s="3" t="n">
-        <v>275</v>
+        <v>48</v>
       </c>
       <c r="AZ16" s="3" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="BA16" s="4" t="inlineStr">
         <is>
-          <t>light wind</t>
+          <t>humid</t>
         </is>
       </c>
       <c r="BB16" s="3" t="n">
-        <v>375</v>
+        <v>404</v>
       </c>
       <c r="BC16" s="3" t="n">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="BD16" s="3" t="n">
-        <v>0.226</v>
+        <v>0.257</v>
       </c>
       <c r="BE16" s="3" t="n">
-        <v>0.277</v>
+        <v>0.339</v>
       </c>
       <c r="BF16" s="3" t="n">
-        <v>0.421</v>
+        <v>0.477</v>
       </c>
       <c r="BG16" s="3" t="n">
-        <v>0.698</v>
+        <v>0.8159999999999999</v>
       </c>
       <c r="BH16" s="3" t="n">
-        <v>97</v>
+        <v>300</v>
       </c>
       <c r="BI16" s="3" t="n">
-        <v>0.607</v>
+        <v>0.783</v>
       </c>
       <c r="BJ16" s="3" t="n">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="BK16" s="3" t="n">
         <v>21</v>
       </c>
       <c r="BL16" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BM16" s="3" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="BN16" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="BO16" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="BP16" s="3" t="n">
         <v>45</v>
-      </c>
-      <c r="BO16" s="3" t="n">
-        <v>36</v>
-      </c>
-      <c r="BP16" s="3" t="n">
-        <v>24</v>
       </c>
       <c r="BQ16" s="3" t="n">
         <v>1</v>
       </c>
       <c r="BR16" s="3" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="BS16" s="3" t="n">
-        <v>8.140000000000001</v>
+        <v>8.710000000000001</v>
       </c>
       <c r="BT16" s="3" t="n">
-        <v>7.21</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="BU16" s="3" t="n">
-        <v>7.07</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="BV16" s="3" t="n">
-        <v>1.804</v>
+        <v>2.262</v>
       </c>
       <c r="BW16" s="3" t="n">
-        <v>0.2143</v>
+        <v>0.2787</v>
       </c>
       <c r="BX16" s="3" t="n">
-        <v>0.0893</v>
+        <v>0.1475</v>
       </c>
       <c r="BY16" s="3" t="n">
-        <v>0.0357</v>
+        <v>0.082</v>
       </c>
       <c r="BZ16" s="3" t="n">
-        <v>0.125</v>
+        <v>0.0492</v>
       </c>
       <c r="CA16" s="3" t="n">
-        <v>0.0179</v>
+        <v>0</v>
       </c>
       <c r="CB16" s="3" t="n">
         <v>8</v>
       </c>
       <c r="CC16" s="3" t="n">
-        <v>8.390000000000001</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="CD16" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="CE16" s="3" t="n">
         <v>16</v>
       </c>
       <c r="CF16" s="3" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="CG16" s="3" t="n">
-        <v>0.1799</v>
+        <v>0.1258</v>
       </c>
       <c r="CH16" s="3" t="n">
-        <v>0.0665</v>
+        <v>0.0526</v>
       </c>
       <c r="CI16" s="3" t="n">
-        <v>0.005</v>
+        <v>0.0025</v>
       </c>
       <c r="CJ16" s="3" t="n">
-        <v>0.0507</v>
+        <v>0.0649</v>
       </c>
       <c r="CK16" s="3" t="n">
-        <v>0.0586</v>
+        <v>0.079</v>
       </c>
       <c r="CL16" s="3" t="n">
-        <v>0.0054</v>
+        <v>0.0061</v>
       </c>
       <c r="CM16" s="3" t="n">
-        <v>0.1388</v>
+        <v>0.1217</v>
       </c>
       <c r="CN16" s="3" t="n">
-        <v>0.1268</v>
+        <v>0.1243</v>
       </c>
       <c r="CO16" s="3" t="n">
-        <v>0.0105</v>
+        <v>0.0142</v>
       </c>
       <c r="CP16" s="4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -5821,28 +5821,28 @@
         <v>10.16</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>9.9</v>
+        <v>9.91</v>
       </c>
       <c r="L17" s="5" t="n">
-        <v>82.40000000000001</v>
+        <v>82.3</v>
       </c>
       <c r="M17" s="5" t="n">
-        <v>74.09999999999999</v>
+        <v>74</v>
       </c>
       <c r="N17" s="5" t="n">
-        <v>74.09999999999999</v>
+        <v>74</v>
       </c>
       <c r="O17" s="5" t="n">
-        <v>71.2</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="P17" s="5" t="n">
-        <v>71.2</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="Q17" s="5" t="n">
-        <v>60.8</v>
+        <v>60.7</v>
       </c>
       <c r="R17" s="5" t="n">
-        <v>60.8</v>
+        <v>60.7</v>
       </c>
       <c r="S17" s="6" t="n">
         <v>57.4</v>
@@ -5851,10 +5851,10 @@
         <v>57.4</v>
       </c>
       <c r="U17" s="7" t="n">
-        <v>51.1</v>
+        <v>51</v>
       </c>
       <c r="V17" s="7" t="n">
-        <v>51.1</v>
+        <v>51</v>
       </c>
       <c r="W17" s="7" t="n">
         <v>46.4</v>
@@ -5869,7 +5869,7 @@
         <v>42.9</v>
       </c>
       <c r="AA17" s="3" t="n">
-        <v>248.47</v>
+        <v>248.53</v>
       </c>
       <c r="AB17" s="4" t="inlineStr">
         <is>
@@ -5956,7 +5956,7 @@
         <v>332</v>
       </c>
       <c r="AZ17" s="3" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="BA17" s="4" t="inlineStr">
         <is>
@@ -6045,7 +6045,7 @@
         <v>8</v>
       </c>
       <c r="CC17" s="3" t="n">
-        <v>8.24</v>
+        <v>8.26</v>
       </c>
       <c r="CD17" s="3" t="n">
         <v>3</v>
@@ -6441,16 +6441,16 @@
         <v>10.03</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>10.02</v>
+        <v>10.04</v>
       </c>
       <c r="L19" s="5" t="n">
         <v>83</v>
       </c>
       <c r="M19" s="5" t="n">
-        <v>75.7</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="N19" s="5" t="n">
-        <v>75.7</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="O19" s="5" t="n">
         <v>71</v>
@@ -6477,10 +6477,10 @@
         <v>49.6</v>
       </c>
       <c r="W19" s="7" t="n">
-        <v>45.2</v>
+        <v>45.3</v>
       </c>
       <c r="X19" s="7" t="n">
-        <v>45.2</v>
+        <v>45.3</v>
       </c>
       <c r="Y19" s="7" t="n">
         <v>41.4</v>
@@ -6489,7 +6489,7 @@
         <v>41.4</v>
       </c>
       <c r="AA19" s="3" t="n">
-        <v>244.4</v>
+        <v>244.55</v>
       </c>
       <c r="AB19" s="4" t="inlineStr">
         <is>
@@ -6657,7 +6657,7 @@
         <v>7</v>
       </c>
       <c r="CC19" s="3" t="n">
-        <v>8.369999999999999</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="CD19" s="3" t="n">
         <v>4</v>
@@ -6747,16 +6747,16 @@
         <v>9.800000000000001</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>9.5</v>
+        <v>9.51</v>
       </c>
       <c r="L20" s="5" t="n">
         <v>80.8</v>
       </c>
       <c r="M20" s="5" t="n">
-        <v>73.09999999999999</v>
+        <v>73</v>
       </c>
       <c r="N20" s="5" t="n">
-        <v>73.09999999999999</v>
+        <v>73</v>
       </c>
       <c r="O20" s="5" t="n">
         <v>68</v>
@@ -6777,25 +6777,25 @@
         <v>54</v>
       </c>
       <c r="U20" s="7" t="n">
-        <v>47.1</v>
+        <v>47.2</v>
       </c>
       <c r="V20" s="7" t="n">
-        <v>47.1</v>
+        <v>47.2</v>
       </c>
       <c r="W20" s="7" t="n">
-        <v>42.7</v>
+        <v>42.8</v>
       </c>
       <c r="X20" s="7" t="n">
-        <v>42.7</v>
+        <v>42.8</v>
       </c>
       <c r="Y20" s="9" t="n">
-        <v>38.9</v>
+        <v>39</v>
       </c>
       <c r="Z20" s="9" t="n">
-        <v>38.9</v>
+        <v>39</v>
       </c>
       <c r="AA20" s="3" t="n">
-        <v>243.01</v>
+        <v>243.1</v>
       </c>
       <c r="AB20" s="4" t="inlineStr">
         <is>
@@ -6882,7 +6882,7 @@
         <v>81</v>
       </c>
       <c r="AZ20" s="3" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="BA20" s="4" t="inlineStr">
         <is>
@@ -6971,7 +6971,7 @@
         <v>7</v>
       </c>
       <c r="CC20" s="3" t="n">
-        <v>8.17</v>
+        <v>8.18</v>
       </c>
       <c r="CD20" s="3" t="n">
         <v>3</v>
@@ -7061,16 +7061,16 @@
         <v>9.789999999999999</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>9.4</v>
+        <v>9.41</v>
       </c>
       <c r="L21" s="5" t="n">
-        <v>82.40000000000001</v>
+        <v>82.5</v>
       </c>
       <c r="M21" s="5" t="n">
-        <v>74.59999999999999</v>
+        <v>74.7</v>
       </c>
       <c r="N21" s="5" t="n">
-        <v>74.59999999999999</v>
+        <v>74.7</v>
       </c>
       <c r="O21" s="5" t="n">
         <v>70.5</v>
@@ -7109,7 +7109,7 @@
         <v>39.9</v>
       </c>
       <c r="AA21" s="3" t="n">
-        <v>242.37</v>
+        <v>242.44</v>
       </c>
       <c r="AB21" s="4" t="inlineStr">
         <is>
@@ -7196,7 +7196,7 @@
         <v>143</v>
       </c>
       <c r="AZ21" s="3" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="BA21" s="4" t="inlineStr">
         <is>
@@ -7375,7 +7375,7 @@
         <v>9.91</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>9.98</v>
+        <v>9.99</v>
       </c>
       <c r="L22" s="5" t="n">
         <v>83.8</v>
@@ -7411,19 +7411,19 @@
         <v>51.4</v>
       </c>
       <c r="W22" s="7" t="n">
-        <v>46.3</v>
+        <v>46.4</v>
       </c>
       <c r="X22" s="7" t="n">
-        <v>46.3</v>
+        <v>46.4</v>
       </c>
       <c r="Y22" s="7" t="n">
-        <v>42.7</v>
+        <v>42.8</v>
       </c>
       <c r="Z22" s="7" t="n">
-        <v>42.7</v>
+        <v>42.8</v>
       </c>
       <c r="AA22" s="3" t="n">
-        <v>242.28</v>
+        <v>242.36</v>
       </c>
       <c r="AB22" s="4" t="inlineStr">
         <is>
@@ -7591,7 +7591,7 @@
         <v>8</v>
       </c>
       <c r="CC22" s="3" t="n">
-        <v>8.109999999999999</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="CD22" s="3" t="n">
         <v>4</v>
@@ -7678,13 +7678,13 @@
         </is>
       </c>
       <c r="J23" s="3" t="n">
-        <v>9.27</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>9.09</v>
+        <v>9.08</v>
       </c>
       <c r="L23" s="5" t="n">
-        <v>81.7</v>
+        <v>81.8</v>
       </c>
       <c r="M23" s="5" t="n">
         <v>74.40000000000001</v>
@@ -7693,28 +7693,28 @@
         <v>74.40000000000001</v>
       </c>
       <c r="O23" s="5" t="n">
-        <v>69.5</v>
+        <v>69.7</v>
       </c>
       <c r="P23" s="5" t="n">
-        <v>69.5</v>
+        <v>69.7</v>
       </c>
       <c r="Q23" s="5" t="n">
-        <v>58.5</v>
+        <v>58.9</v>
       </c>
       <c r="R23" s="5" t="n">
-        <v>58.5</v>
+        <v>58.9</v>
       </c>
       <c r="S23" s="6" t="n">
-        <v>54.5</v>
+        <v>54.8</v>
       </c>
       <c r="T23" s="7" t="n">
-        <v>54.5</v>
+        <v>54.8</v>
       </c>
       <c r="U23" s="7" t="n">
-        <v>46.6</v>
+        <v>46.7</v>
       </c>
       <c r="V23" s="7" t="n">
-        <v>46.6</v>
+        <v>46.7</v>
       </c>
       <c r="W23" s="7" t="n">
         <v>41.9</v>
@@ -7723,13 +7723,13 @@
         <v>41.9</v>
       </c>
       <c r="Y23" s="9" t="n">
-        <v>37.2</v>
+        <v>37.4</v>
       </c>
       <c r="Z23" s="9" t="n">
-        <v>37.2</v>
+        <v>37.4</v>
       </c>
       <c r="AA23" s="3" t="n">
-        <v>240.9</v>
+        <v>241.02</v>
       </c>
       <c r="AB23" s="4" t="inlineStr">
         <is>
@@ -7842,10 +7842,10 @@
         <v>0.802</v>
       </c>
       <c r="BH23" s="3" t="n">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="BI23" s="3" t="n">
-        <v>0.803</v>
+        <v>0.8159999999999999</v>
       </c>
       <c r="BJ23" s="3" t="n">
         <v>72</v>
@@ -7905,7 +7905,7 @@
         <v>7</v>
       </c>
       <c r="CC23" s="3" t="n">
-        <v>7.6</v>
+        <v>7.54</v>
       </c>
       <c r="CD23" s="3" t="n">
         <v>3</v>
@@ -7917,7 +7917,7 @@
         <v>20</v>
       </c>
       <c r="CG23" s="3" t="n">
-        <v>0.1574</v>
+        <v>0.1585</v>
       </c>
       <c r="CH23" s="3" t="n">
         <v>0.0541</v>
@@ -7929,16 +7929,16 @@
         <v>0.038</v>
       </c>
       <c r="CK23" s="3" t="n">
-        <v>0.1268</v>
+        <v>0.1266</v>
       </c>
       <c r="CL23" s="3" t="n">
         <v>0.0136</v>
       </c>
       <c r="CM23" s="3" t="n">
-        <v>0.1303</v>
+        <v>0.1302</v>
       </c>
       <c r="CN23" s="3" t="n">
-        <v>0.1398</v>
+        <v>0.141</v>
       </c>
       <c r="CO23" s="3" t="n">
         <v>0.0111</v>
@@ -7998,7 +7998,7 @@
         <v>9.82</v>
       </c>
       <c r="L24" s="5" t="n">
-        <v>83.3</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="M24" s="5" t="n">
         <v>74.59999999999999</v>
@@ -8031,19 +8031,19 @@
         <v>50.5</v>
       </c>
       <c r="W24" s="7" t="n">
-        <v>45.6</v>
+        <v>45.5</v>
       </c>
       <c r="X24" s="7" t="n">
-        <v>45.6</v>
+        <v>45.5</v>
       </c>
       <c r="Y24" s="7" t="n">
-        <v>42.2</v>
+        <v>42.1</v>
       </c>
       <c r="Z24" s="7" t="n">
-        <v>42.2</v>
+        <v>42.1</v>
       </c>
       <c r="AA24" s="3" t="n">
-        <v>238.52</v>
+        <v>238.51</v>
       </c>
       <c r="AB24" s="4" t="inlineStr">
         <is>
@@ -8219,7 +8219,7 @@
         <v>8</v>
       </c>
       <c r="CC24" s="3" t="n">
-        <v>8.15</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="CD24" s="3" t="n">
         <v>3</v>
@@ -8351,10 +8351,10 @@
         <v>45.1</v>
       </c>
       <c r="Y25" s="7" t="n">
-        <v>42.4</v>
+        <v>42.5</v>
       </c>
       <c r="Z25" s="7" t="n">
-        <v>42.4</v>
+        <v>42.5</v>
       </c>
       <c r="AA25" s="3" t="n">
         <v>238.14</v>
@@ -8412,13 +8412,13 @@
         <v>0.0476</v>
       </c>
       <c r="AP25" s="3" t="n">
-        <v>5.46</v>
+        <v>5.47</v>
       </c>
       <c r="AQ25" s="3" t="n">
         <v>1.52</v>
       </c>
       <c r="AR25" s="3" t="n">
-        <v>0.2557</v>
+        <v>0.2555</v>
       </c>
       <c r="AS25" s="3" t="n">
         <v>0.0346</v>
@@ -8557,7 +8557,7 @@
         <v>0.0511</v>
       </c>
       <c r="CK25" s="3" t="n">
-        <v>0.0498</v>
+        <v>0.0499</v>
       </c>
       <c r="CL25" s="3" t="n">
         <v>0.0056</v>
@@ -8641,10 +8641,10 @@
         <v>60.8</v>
       </c>
       <c r="Q26" s="6" t="n">
-        <v>51</v>
+        <v>51.1</v>
       </c>
       <c r="R26" s="7" t="n">
-        <v>51</v>
+        <v>51.1</v>
       </c>
       <c r="S26" s="7" t="n">
         <v>48.1</v>
@@ -8665,10 +8665,10 @@
         <v>38.7</v>
       </c>
       <c r="Y26" s="9" t="n">
-        <v>36.3</v>
+        <v>36.4</v>
       </c>
       <c r="Z26" s="9" t="n">
-        <v>36.3</v>
+        <v>36.4</v>
       </c>
       <c r="AA26" s="3" t="n">
         <v>236.73</v>
@@ -8839,7 +8839,7 @@
         <v>6</v>
       </c>
       <c r="CC26" s="3" t="n">
-        <v>8.630000000000001</v>
+        <v>8.640000000000001</v>
       </c>
       <c r="CD26" s="3" t="n">
         <v>2</v>
@@ -9064,7 +9064,7 @@
         <v>286</v>
       </c>
       <c r="AZ27" s="3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="BA27" s="4" t="inlineStr">
         <is>
@@ -9211,22 +9211,22 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Trevor Larnach</t>
+          <t>James Wood</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>LAA</t>
+          <t>NYY</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>LAA @ MIN</t>
+          <t>NYY @ WSH</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
@@ -9236,62 +9236,62 @@
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>LF</t>
+          <t>RF</t>
         </is>
       </c>
       <c r="J28" s="3" t="n">
-        <v>9.630000000000001</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>9.699999999999999</v>
+        <v>7.95</v>
       </c>
       <c r="L28" s="5" t="n">
-        <v>85.2</v>
+        <v>72.2</v>
       </c>
       <c r="M28" s="5" t="n">
-        <v>76.8</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="N28" s="5" t="n">
-        <v>76.8</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="O28" s="5" t="n">
-        <v>73.40000000000001</v>
+        <v>59.5</v>
       </c>
       <c r="P28" s="5" t="n">
-        <v>73.40000000000001</v>
-      </c>
-      <c r="Q28" s="5" t="n">
-        <v>62.6</v>
-      </c>
-      <c r="R28" s="5" t="n">
-        <v>62.6</v>
-      </c>
-      <c r="S28" s="5" t="n">
-        <v>58.5</v>
-      </c>
-      <c r="T28" s="5" t="n">
-        <v>58.5</v>
-      </c>
-      <c r="U28" s="6" t="n">
-        <v>50.5</v>
-      </c>
-      <c r="V28" s="7" t="n">
-        <v>50.5</v>
-      </c>
-      <c r="W28" s="7" t="n">
-        <v>44.9</v>
-      </c>
-      <c r="X28" s="7" t="n">
-        <v>44.9</v>
-      </c>
-      <c r="Y28" s="7" t="n">
-        <v>41</v>
-      </c>
-      <c r="Z28" s="7" t="n">
-        <v>41</v>
+        <v>59.5</v>
+      </c>
+      <c r="Q28" s="6" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="R28" s="7" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="S28" s="7" t="n">
+        <v>45.8</v>
+      </c>
+      <c r="T28" s="7" t="n">
+        <v>45.8</v>
+      </c>
+      <c r="U28" s="9" t="n">
+        <v>38.7</v>
+      </c>
+      <c r="V28" s="9" t="n">
+        <v>38.7</v>
+      </c>
+      <c r="W28" s="9" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="X28" s="9" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="Y28" s="9" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="Z28" s="9" t="n">
+        <v>31.4</v>
       </c>
       <c r="AA28" s="3" t="n">
-        <v>234.73</v>
+        <v>234.76</v>
       </c>
       <c r="AB28" s="4" t="inlineStr">
         <is>
@@ -9300,14 +9300,14 @@
       </c>
       <c r="AC28" s="8" t="inlineStr">
         <is>
-          <t>Forecast 9.6 FS | Sim 9.7</t>
+          <t>Forecast 8.8 FS | Sim 8.0</t>
         </is>
       </c>
       <c r="AD28" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AE28" s="3" t="n">
-        <v>4.52</v>
+        <v>5.13</v>
       </c>
       <c r="AF28" s="4" t="inlineStr">
         <is>
@@ -9315,14 +9315,14 @@
         </is>
       </c>
       <c r="AG28" s="3" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="AH28" s="3" t="n">
         <v>1.04</v>
       </c>
       <c r="AI28" s="4" t="inlineStr">
         <is>
-          <t>Ryan Johnson</t>
+          <t>Cam Schlittler</t>
         </is>
       </c>
       <c r="AJ28" s="4" t="inlineStr">
@@ -9331,54 +9331,54 @@
         </is>
       </c>
       <c r="AK28" s="3" t="n">
-        <v>6.99</v>
+        <v>2.01</v>
       </c>
       <c r="AL28" s="3" t="n">
-        <v>1.55</v>
+        <v>0.93</v>
       </c>
       <c r="AM28" s="3" t="n">
-        <v>0.2595</v>
+        <v>0.1878</v>
       </c>
       <c r="AN28" s="3" t="n">
-        <v>0.0611</v>
+        <v>0.0226</v>
       </c>
       <c r="AO28" s="3" t="n">
-        <v>0.07630000000000001</v>
+        <v>0.0475</v>
       </c>
       <c r="AP28" s="3" t="n">
-        <v>4.65</v>
+        <v>3.4</v>
       </c>
       <c r="AQ28" s="3" t="n">
-        <v>1.4</v>
+        <v>1.19</v>
       </c>
       <c r="AR28" s="3" t="n">
-        <v>0.2052</v>
+        <v>0.2049</v>
       </c>
       <c r="AS28" s="3" t="n">
-        <v>0.028</v>
+        <v>0.0267</v>
       </c>
       <c r="AT28" s="4" t="inlineStr">
         <is>
-          <t>Target Field</t>
+          <t>Nationals Park</t>
         </is>
       </c>
       <c r="AU28" s="3" t="n">
-        <v>0.98</v>
+        <v>1</v>
       </c>
       <c r="AV28" s="3" t="n">
         <v>1.03</v>
       </c>
       <c r="AW28" s="3" t="n">
-        <v>88.3</v>
+        <v>84.2</v>
       </c>
       <c r="AX28" s="3" t="n">
-        <v>5.9</v>
+        <v>4.8</v>
       </c>
       <c r="AY28" s="3" t="n">
-        <v>191</v>
+        <v>332</v>
       </c>
       <c r="AZ28" s="3" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="BA28" s="4" t="inlineStr">
         <is>
@@ -9386,128 +9386,128 @@
         </is>
       </c>
       <c r="BB28" s="3" t="n">
-        <v>284</v>
+        <v>445</v>
       </c>
       <c r="BC28" s="3" t="n">
-        <v>246</v>
+        <v>362</v>
       </c>
       <c r="BD28" s="3" t="n">
-        <v>0.285</v>
+        <v>0.273</v>
       </c>
       <c r="BE28" s="3" t="n">
-        <v>0.378</v>
+        <v>0.404</v>
       </c>
       <c r="BF28" s="3" t="n">
-        <v>0.439</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="BG28" s="3" t="n">
-        <v>0.8169999999999999</v>
+        <v>0.962</v>
       </c>
       <c r="BH28" s="3" t="n">
-        <v>250</v>
+        <v>296</v>
       </c>
       <c r="BI28" s="3" t="n">
-        <v>0.833</v>
+        <v>0.997</v>
       </c>
       <c r="BJ28" s="3" t="n">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="BK28" s="3" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="BL28" s="3" t="n">
         <v>1</v>
       </c>
       <c r="BM28" s="3" t="n">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="BN28" s="3" t="n">
-        <v>42</v>
+        <v>87</v>
       </c>
       <c r="BO28" s="3" t="n">
-        <v>30</v>
+        <v>62</v>
       </c>
       <c r="BP28" s="3" t="n">
-        <v>34</v>
+        <v>77</v>
       </c>
       <c r="BQ28" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BR28" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="BS28" s="3" t="n">
+        <v>19.14</v>
+      </c>
+      <c r="BT28" s="3" t="n">
+        <v>14.86</v>
+      </c>
+      <c r="BU28" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="BV28" s="3" t="n">
+        <v>3.059</v>
+      </c>
+      <c r="BW28" s="3" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="BX28" s="3" t="n">
+        <v>0.1618</v>
+      </c>
+      <c r="BY28" s="3" t="n">
+        <v>0.0882</v>
+      </c>
+      <c r="BZ28" s="3" t="n">
+        <v>0.2353</v>
+      </c>
+      <c r="CA28" s="3" t="n">
+        <v>0.0294</v>
+      </c>
+      <c r="CB28" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="CC28" s="3" t="n">
+        <v>7.67</v>
+      </c>
+      <c r="CD28" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="BS28" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="BT28" s="3" t="n">
-        <v>7.07</v>
-      </c>
-      <c r="BU28" s="3" t="n">
-        <v>7.53</v>
-      </c>
-      <c r="BV28" s="3" t="n">
-        <v>1.868</v>
-      </c>
-      <c r="BW28" s="3" t="n">
-        <v>0.2642</v>
-      </c>
-      <c r="BX28" s="3" t="n">
-        <v>0.1321</v>
-      </c>
-      <c r="BY28" s="3" t="n">
-        <v>0.0189</v>
-      </c>
-      <c r="BZ28" s="3" t="n">
-        <v>0.1132</v>
-      </c>
-      <c r="CA28" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CB28" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="CC28" s="3" t="n">
-        <v>7.71</v>
-      </c>
-      <c r="CD28" s="3" t="n">
-        <v>4</v>
-      </c>
       <c r="CE28" s="3" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="CF28" s="3" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="CG28" s="3" t="n">
-        <v>0.1787</v>
+        <v>0.096</v>
       </c>
       <c r="CH28" s="3" t="n">
-        <v>0.0711</v>
+        <v>0.0396</v>
       </c>
       <c r="CI28" s="3" t="n">
-        <v>0.0042</v>
+        <v>0.0033</v>
       </c>
       <c r="CJ28" s="3" t="n">
-        <v>0.0405</v>
+        <v>0.0369</v>
       </c>
       <c r="CK28" s="3" t="n">
-        <v>0.1064</v>
+        <v>0.1029</v>
       </c>
       <c r="CL28" s="3" t="n">
-        <v>0.0109</v>
+        <v>0.0065</v>
       </c>
       <c r="CM28" s="3" t="n">
-        <v>0.1268</v>
+        <v>0.1514</v>
       </c>
       <c r="CN28" s="3" t="n">
-        <v>0.1325</v>
+        <v>0.1071</v>
       </c>
       <c r="CO28" s="3" t="n">
-        <v>0.0092</v>
+        <v>0.019</v>
       </c>
       <c r="CP28" s="4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -9525,22 +9525,22 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>James Wood</t>
+          <t>Trevor Larnach</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>WSH</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>NYY</t>
+          <t>LAA</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>NYY @ WSH</t>
+          <t>LAA @ MIN</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
@@ -9550,62 +9550,62 @@
       </c>
       <c r="I29" s="4" t="inlineStr">
         <is>
-          <t>RF</t>
+          <t>LF</t>
         </is>
       </c>
       <c r="J29" s="3" t="n">
-        <v>8.779999999999999</v>
+        <v>9.630000000000001</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>7.94</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="L29" s="5" t="n">
-        <v>72.40000000000001</v>
+        <v>85.2</v>
       </c>
       <c r="M29" s="5" t="n">
-        <v>65.40000000000001</v>
+        <v>76.8</v>
       </c>
       <c r="N29" s="5" t="n">
-        <v>65.40000000000001</v>
+        <v>76.8</v>
       </c>
       <c r="O29" s="5" t="n">
-        <v>59.5</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="P29" s="5" t="n">
-        <v>59.5</v>
-      </c>
-      <c r="Q29" s="6" t="n">
-        <v>49.2</v>
-      </c>
-      <c r="R29" s="7" t="n">
-        <v>49.2</v>
-      </c>
-      <c r="S29" s="7" t="n">
-        <v>45.8</v>
-      </c>
-      <c r="T29" s="7" t="n">
-        <v>45.8</v>
-      </c>
-      <c r="U29" s="9" t="n">
-        <v>38.6</v>
-      </c>
-      <c r="V29" s="9" t="n">
-        <v>38.6</v>
-      </c>
-      <c r="W29" s="9" t="n">
-        <v>35.4</v>
-      </c>
-      <c r="X29" s="9" t="n">
-        <v>35.4</v>
-      </c>
-      <c r="Y29" s="9" t="n">
-        <v>31.3</v>
-      </c>
-      <c r="Z29" s="9" t="n">
-        <v>31.3</v>
+        <v>73.40000000000001</v>
+      </c>
+      <c r="Q29" s="5" t="n">
+        <v>62.6</v>
+      </c>
+      <c r="R29" s="5" t="n">
+        <v>62.6</v>
+      </c>
+      <c r="S29" s="5" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="T29" s="5" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="U29" s="6" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="V29" s="7" t="n">
+        <v>50.5</v>
+      </c>
+      <c r="W29" s="7" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="X29" s="7" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="Y29" s="7" t="n">
+        <v>41</v>
+      </c>
+      <c r="Z29" s="7" t="n">
+        <v>41</v>
       </c>
       <c r="AA29" s="3" t="n">
-        <v>234.68</v>
+        <v>234.73</v>
       </c>
       <c r="AB29" s="4" t="inlineStr">
         <is>
@@ -9614,14 +9614,14 @@
       </c>
       <c r="AC29" s="8" t="inlineStr">
         <is>
-          <t>Forecast 8.8 FS | Sim 7.9</t>
+          <t>Forecast 9.6 FS | Sim 9.7</t>
         </is>
       </c>
       <c r="AD29" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="AE29" s="3" t="n">
-        <v>5.13</v>
+        <v>4.52</v>
       </c>
       <c r="AF29" s="4" t="inlineStr">
         <is>
@@ -9629,14 +9629,14 @@
         </is>
       </c>
       <c r="AG29" s="3" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="AH29" s="3" t="n">
         <v>1.04</v>
       </c>
       <c r="AI29" s="4" t="inlineStr">
         <is>
-          <t>Cam Schlittler</t>
+          <t>Ryan Johnson</t>
         </is>
       </c>
       <c r="AJ29" s="4" t="inlineStr">
@@ -9645,54 +9645,54 @@
         </is>
       </c>
       <c r="AK29" s="3" t="n">
-        <v>2.01</v>
+        <v>6.99</v>
       </c>
       <c r="AL29" s="3" t="n">
-        <v>0.93</v>
+        <v>1.55</v>
       </c>
       <c r="AM29" s="3" t="n">
-        <v>0.1878</v>
+        <v>0.2595</v>
       </c>
       <c r="AN29" s="3" t="n">
-        <v>0.0226</v>
+        <v>0.0611</v>
       </c>
       <c r="AO29" s="3" t="n">
-        <v>0.0475</v>
+        <v>0.07630000000000001</v>
       </c>
       <c r="AP29" s="3" t="n">
-        <v>3.4</v>
+        <v>4.65</v>
       </c>
       <c r="AQ29" s="3" t="n">
-        <v>1.19</v>
+        <v>1.4</v>
       </c>
       <c r="AR29" s="3" t="n">
-        <v>0.2049</v>
+        <v>0.2052</v>
       </c>
       <c r="AS29" s="3" t="n">
-        <v>0.0267</v>
+        <v>0.028</v>
       </c>
       <c r="AT29" s="4" t="inlineStr">
         <is>
-          <t>Nationals Park</t>
+          <t>Target Field</t>
         </is>
       </c>
       <c r="AU29" s="3" t="n">
-        <v>1</v>
+        <v>0.98</v>
       </c>
       <c r="AV29" s="3" t="n">
         <v>1.03</v>
       </c>
       <c r="AW29" s="3" t="n">
-        <v>84.2</v>
+        <v>88.3</v>
       </c>
       <c r="AX29" s="3" t="n">
-        <v>4.8</v>
+        <v>5.9</v>
       </c>
       <c r="AY29" s="3" t="n">
-        <v>332</v>
+        <v>191</v>
       </c>
       <c r="AZ29" s="3" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="BA29" s="4" t="inlineStr">
         <is>
@@ -9700,128 +9700,128 @@
         </is>
       </c>
       <c r="BB29" s="3" t="n">
-        <v>445</v>
+        <v>284</v>
       </c>
       <c r="BC29" s="3" t="n">
-        <v>362</v>
+        <v>246</v>
       </c>
       <c r="BD29" s="3" t="n">
-        <v>0.273</v>
+        <v>0.285</v>
       </c>
       <c r="BE29" s="3" t="n">
-        <v>0.404</v>
+        <v>0.378</v>
       </c>
       <c r="BF29" s="3" t="n">
-        <v>0.5580000000000001</v>
+        <v>0.439</v>
       </c>
       <c r="BG29" s="3" t="n">
-        <v>0.962</v>
+        <v>0.8169999999999999</v>
       </c>
       <c r="BH29" s="3" t="n">
-        <v>296</v>
+        <v>250</v>
       </c>
       <c r="BI29" s="3" t="n">
-        <v>0.997</v>
+        <v>0.833</v>
       </c>
       <c r="BJ29" s="3" t="n">
-        <v>99</v>
+        <v>70</v>
       </c>
       <c r="BK29" s="3" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="BL29" s="3" t="n">
         <v>1</v>
       </c>
       <c r="BM29" s="3" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="BN29" s="3" t="n">
-        <v>87</v>
+        <v>42</v>
       </c>
       <c r="BO29" s="3" t="n">
-        <v>62</v>
+        <v>30</v>
       </c>
       <c r="BP29" s="3" t="n">
-        <v>77</v>
+        <v>34</v>
       </c>
       <c r="BQ29" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="BR29" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="BS29" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="BT29" s="3" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="BU29" s="3" t="n">
+        <v>7.53</v>
+      </c>
+      <c r="BV29" s="3" t="n">
+        <v>1.868</v>
+      </c>
+      <c r="BW29" s="3" t="n">
+        <v>0.2642</v>
+      </c>
+      <c r="BX29" s="3" t="n">
+        <v>0.1321</v>
+      </c>
+      <c r="BY29" s="3" t="n">
+        <v>0.0189</v>
+      </c>
+      <c r="BZ29" s="3" t="n">
+        <v>0.1132</v>
+      </c>
+      <c r="CA29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CB29" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="CC29" s="3" t="n">
+        <v>7.71</v>
+      </c>
+      <c r="CD29" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="BR29" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="BS29" s="3" t="n">
-        <v>19.14</v>
-      </c>
-      <c r="BT29" s="3" t="n">
-        <v>14.86</v>
-      </c>
-      <c r="BU29" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="BV29" s="3" t="n">
-        <v>3.059</v>
-      </c>
-      <c r="BW29" s="3" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="BX29" s="3" t="n">
-        <v>0.1618</v>
-      </c>
-      <c r="BY29" s="3" t="n">
-        <v>0.0882</v>
-      </c>
-      <c r="BZ29" s="3" t="n">
-        <v>0.2353</v>
-      </c>
-      <c r="CA29" s="3" t="n">
-        <v>0.0294</v>
-      </c>
-      <c r="CB29" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="CC29" s="3" t="n">
-        <v>7.66</v>
-      </c>
-      <c r="CD29" s="3" t="n">
-        <v>2</v>
-      </c>
       <c r="CE29" s="3" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="CF29" s="3" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="CG29" s="3" t="n">
-        <v>0.096</v>
+        <v>0.1787</v>
       </c>
       <c r="CH29" s="3" t="n">
-        <v>0.0396</v>
+        <v>0.0711</v>
       </c>
       <c r="CI29" s="3" t="n">
-        <v>0.0033</v>
+        <v>0.0042</v>
       </c>
       <c r="CJ29" s="3" t="n">
-        <v>0.0369</v>
+        <v>0.0405</v>
       </c>
       <c r="CK29" s="3" t="n">
-        <v>0.1029</v>
+        <v>0.1064</v>
       </c>
       <c r="CL29" s="3" t="n">
-        <v>0.0065</v>
+        <v>0.0109</v>
       </c>
       <c r="CM29" s="3" t="n">
-        <v>0.1514</v>
+        <v>0.1268</v>
       </c>
       <c r="CN29" s="3" t="n">
-        <v>0.1071</v>
+        <v>0.1325</v>
       </c>
       <c r="CO29" s="3" t="n">
-        <v>0.019</v>
+        <v>0.0092</v>
       </c>
       <c r="CP29" s="4" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -9877,28 +9877,28 @@
         <v>78.5</v>
       </c>
       <c r="M30" s="5" t="n">
-        <v>69.5</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="N30" s="5" t="n">
-        <v>69.5</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="O30" s="5" t="n">
-        <v>66.2</v>
+        <v>66.3</v>
       </c>
       <c r="P30" s="5" t="n">
-        <v>66.2</v>
+        <v>66.3</v>
       </c>
       <c r="Q30" s="6" t="n">
-        <v>56.2</v>
+        <v>56.3</v>
       </c>
       <c r="R30" s="7" t="n">
-        <v>56.2</v>
+        <v>56.3</v>
       </c>
       <c r="S30" s="7" t="n">
-        <v>52.9</v>
+        <v>53</v>
       </c>
       <c r="T30" s="7" t="n">
-        <v>52.9</v>
+        <v>53</v>
       </c>
       <c r="U30" s="7" t="n">
         <v>47.2</v>
@@ -9913,13 +9913,13 @@
         <v>43.1</v>
       </c>
       <c r="Y30" s="7" t="n">
-        <v>40.2</v>
+        <v>40.3</v>
       </c>
       <c r="Z30" s="7" t="n">
-        <v>40.2</v>
+        <v>40.3</v>
       </c>
       <c r="AA30" s="3" t="n">
-        <v>234.65</v>
+        <v>234.66</v>
       </c>
       <c r="AB30" s="4" t="inlineStr">
         <is>
@@ -10006,7 +10006,7 @@
         <v>48</v>
       </c>
       <c r="AZ30" s="3" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="BA30" s="4" t="inlineStr">
         <is>
@@ -10095,13 +10095,13 @@
         <v>7</v>
       </c>
       <c r="CC30" s="3" t="n">
-        <v>8.6</v>
+        <v>8.59</v>
       </c>
       <c r="CD30" s="3" t="n">
         <v>3</v>
       </c>
       <c r="CE30" s="3" t="n">
-        <v>14</v>
+        <v>14.25</v>
       </c>
       <c r="CF30" s="3" t="n">
         <v>21</v>

</xml_diff>